<commit_message>
points clear for s5
</commit_message>
<xml_diff>
--- a/the_alternative_f1/The_Alternative_F1.xlsx
+++ b/the_alternative_f1/The_Alternative_F1.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2462" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3166" uniqueCount="435">
   <si>
     <t>Positions</t>
   </si>
@@ -2840,14 +2840,10 @@
       <c r="C2" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="16">
-        <v>1.0</v>
-      </c>
-      <c r="E2" s="17">
-        <v>16.0</v>
-      </c>
+      <c r="D2" s="16"/>
+      <c r="E2" s="17"/>
       <c r="F2" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G2" s="19" t="s">
         <v>128</v>
@@ -2860,158 +2856,238 @@
       </c>
       <c r="J2" s="71">
         <f>IFERROR((VLOOKUP(D2,Scoring!$A:$B,2,0))+IF(F2="y",1,0)+IF(G2="y",1,0)+IF(H2="y",1,0)+IF(I2="y",1,0),0)</f>
-        <v>26</v>
-      </c>
-      <c r="K2" s="16">
-        <v>2.0</v>
-      </c>
-      <c r="L2" s="17">
-        <v>1.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K2" s="16"/>
+      <c r="L2" s="17"/>
       <c r="M2" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="N2" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O2" s="20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="P2" s="21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q2" s="71">
         <f>IFERROR((VLOOKUP(K2,Scoring!$A:$B,2,0))+IF(M2="y",1,0)+IF(N2="y",1,0)+IF(O2="y",1,0)+IF(P2="y",1,0),0)</f>
-        <v>22</v>
-      </c>
-      <c r="R2" s="16">
-        <v>16.0</v>
-      </c>
-      <c r="S2" s="17">
-        <v>16.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R2" s="16"/>
+      <c r="S2" s="17"/>
       <c r="T2" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="U2" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="V2" s="20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="W2" s="21" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="X2" s="71">
         <f>IFERROR((VLOOKUP(R2,Scoring!$A:$B,2,0))+IF(T2="y",1,0)+IF(U2="y",1,0)+IF(V2="y",1,0)+IF(W2="y",1,0),0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="Y2" s="16"/>
       <c r="Z2" s="17"/>
-      <c r="AA2" s="18"/>
-      <c r="AB2" s="19"/>
-      <c r="AC2" s="20"/>
-      <c r="AD2" s="21"/>
+      <c r="AA2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="AE2" s="71">
         <f>IFERROR((VLOOKUP(Y2,Scoring!$A:$B,2,0))+IF(AA2="y",1,0)+IF(AB2="y",1,0)+IF(AC2="y",1,0)+IF(AD2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF2" s="16"/>
       <c r="AG2" s="17"/>
-      <c r="AH2" s="18"/>
-      <c r="AI2" s="19"/>
-      <c r="AJ2" s="20"/>
-      <c r="AK2" s="21"/>
+      <c r="AH2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="AL2" s="71">
         <f>IFERROR((VLOOKUP(AF2,Scoring!$A:$B,2,0))+IF(AH2="y",1,0)+IF(AI2="y",1,0)+IF(AJ2="y",1,0)+IF(AK2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM2" s="16"/>
       <c r="AN2" s="17"/>
-      <c r="AO2" s="18"/>
-      <c r="AP2" s="19"/>
-      <c r="AQ2" s="20"/>
-      <c r="AR2" s="21"/>
+      <c r="AO2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="AS2" s="71">
         <f>IFERROR((VLOOKUP(AM2,Scoring!$A:$B,2,0))+IF(AO2="y",1,0)+IF(AP2="y",1,0)+IF(AQ2="y",1,0)+IF(AR2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT2" s="16"/>
       <c r="AU2" s="17"/>
-      <c r="AV2" s="18"/>
-      <c r="AW2" s="19"/>
-      <c r="AX2" s="20"/>
-      <c r="AY2" s="21"/>
+      <c r="AV2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ2" s="71">
         <f>IFERROR((VLOOKUP(AT2,Scoring!$A:$B,2,0))+IF(AV2="y",1,0)+IF(AW2="y",1,0)+IF(AX2="y",1,0)+IF(AY2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA2" s="16"/>
       <c r="BB2" s="17"/>
-      <c r="BC2" s="18"/>
-      <c r="BD2" s="19"/>
-      <c r="BE2" s="20"/>
-      <c r="BF2" s="21"/>
+      <c r="BC2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="BG2" s="71">
         <f>IFERROR((VLOOKUP(BA2,Scoring!$A:$B,2,0))+IF(BC2="y",1,0)+IF(BD2="y",1,0)+IF(BE2="y",1,0)+IF(BF2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH2" s="16"/>
       <c r="BI2" s="17"/>
-      <c r="BJ2" s="18"/>
-      <c r="BK2" s="19"/>
-      <c r="BL2" s="20"/>
-      <c r="BM2" s="21"/>
+      <c r="BJ2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="BN2" s="71">
         <f>IFERROR((VLOOKUP(BH2,Scoring!$A:$B,2,0))+IF(BJ2="y",1,0)+IF(BK2="y",1,0)+IF(BL2="y",1,0)+IF(BM2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO2" s="16"/>
       <c r="BP2" s="17"/>
-      <c r="BQ2" s="18"/>
-      <c r="BR2" s="19"/>
-      <c r="BS2" s="20"/>
-      <c r="BT2" s="21"/>
+      <c r="BQ2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="BU2" s="71">
         <f>IFERROR((VLOOKUP(BO2,Scoring!$A:$B,2,0))+IF(BQ2="y",1,0)+IF(BR2="y",1,0)+IF(BS2="y",1,0)+IF(BT2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV2" s="16"/>
       <c r="BW2" s="17"/>
-      <c r="BX2" s="18"/>
-      <c r="BY2" s="19"/>
-      <c r="BZ2" s="20"/>
-      <c r="CA2" s="21"/>
+      <c r="BX2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="CB2" s="71">
         <f>IFERROR((VLOOKUP(BV2,Scoring!$A:$B,2,0))+IF(BX2="y",1,0)+IF(BY2="y",1,0)+IF(BZ2="y",1,0)+IF(CA2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC2" s="16"/>
       <c r="CD2" s="17"/>
-      <c r="CE2" s="18"/>
-      <c r="CF2" s="19"/>
-      <c r="CG2" s="20"/>
-      <c r="CH2" s="21"/>
+      <c r="CE2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="CI2" s="71">
         <f>IFERROR((VLOOKUP(CC2,Scoring!$A:$B,2,0))+IF(CE2="y",1,0)+IF(CF2="y",1,0)+IF(CG2="y",1,0)+IF(CH2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ2" s="16"/>
       <c r="CK2" s="17"/>
-      <c r="CL2" s="18"/>
-      <c r="CM2" s="19"/>
-      <c r="CN2" s="20"/>
-      <c r="CO2" s="21"/>
+      <c r="CL2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="CP2" s="71">
         <f>IFERROR((VLOOKUP(CJ2,Scoring!$A:$B,2,0))+IF(CL2="y",1,0)+IF(CM2="y",1,0)+IF(CN2="y",1,0)+IF(CO2="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ2" s="16"/>
       <c r="CR2" s="17"/>
-      <c r="CS2" s="18"/>
-      <c r="CT2" s="19"/>
-      <c r="CU2" s="20"/>
-      <c r="CV2" s="21"/>
+      <c r="CS2" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT2" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU2" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV2" s="21" t="s">
+        <v>128</v>
+      </c>
       <c r="CW2" s="71">
         <f>IFERROR((VLOOKUP(CQ2,Scoring!$A:$B,2,0))+IF(CS2="y",1,0)+IF(CT2="y",1,0)+IF(CU2="y",1,0)+IF(CV2="y",1,0),0)</f>
         <v>0</v>
@@ -3030,17 +3106,13 @@
       <c r="C3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="24">
-        <v>2.0</v>
-      </c>
-      <c r="E3" s="25">
-        <v>15.0</v>
-      </c>
+      <c r="D3" s="24"/>
+      <c r="E3" s="25"/>
       <c r="F3" s="26" t="s">
         <v>128</v>
       </c>
       <c r="G3" s="27" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H3" s="28" t="s">
         <v>128</v>
@@ -3050,14 +3122,10 @@
       </c>
       <c r="J3" s="72">
         <f>IFERROR((VLOOKUP(D3,Scoring!$A:$B,2,0))+IF(F3="y",1,0)+IF(G3="y",1,0)+IF(H3="y",1,0)+IF(I3="y",1,0),0)</f>
-        <v>19</v>
-      </c>
-      <c r="K3" s="24">
-        <v>4.0</v>
-      </c>
-      <c r="L3" s="25">
-        <v>2.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K3" s="24"/>
+      <c r="L3" s="25"/>
       <c r="M3" s="26" t="s">
         <v>128</v>
       </c>
@@ -3072,14 +3140,10 @@
       </c>
       <c r="Q3" s="72">
         <f>IFERROR((VLOOKUP(K3,Scoring!$A:$B,2,0))+IF(M3="y",1,0)+IF(N3="y",1,0)+IF(O3="y",1,0)+IF(P3="y",1,0),0)</f>
-        <v>12</v>
-      </c>
-      <c r="R3" s="24">
-        <v>14.0</v>
-      </c>
-      <c r="S3" s="25">
-        <v>14.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R3" s="24"/>
+      <c r="S3" s="25"/>
       <c r="T3" s="26" t="s">
         <v>128</v>
       </c>
@@ -3094,114 +3158,202 @@
       </c>
       <c r="X3" s="72">
         <f>IFERROR((VLOOKUP(R3,Scoring!$A:$B,2,0))+IF(T3="y",1,0)+IF(U3="y",1,0)+IF(V3="y",1,0)+IF(W3="y",1,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="24"/>
       <c r="Z3" s="25"/>
-      <c r="AA3" s="26"/>
-      <c r="AB3" s="27"/>
-      <c r="AC3" s="28"/>
-      <c r="AD3" s="29"/>
+      <c r="AA3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AE3" s="72">
         <f>IFERROR((VLOOKUP(Y3,Scoring!$A:$B,2,0))+IF(AA3="y",1,0)+IF(AB3="y",1,0)+IF(AC3="y",1,0)+IF(AD3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF3" s="24"/>
       <c r="AG3" s="25"/>
-      <c r="AH3" s="26"/>
-      <c r="AI3" s="27"/>
-      <c r="AJ3" s="28"/>
-      <c r="AK3" s="29"/>
+      <c r="AH3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AL3" s="72">
         <f>IFERROR((VLOOKUP(AF3,Scoring!$A:$B,2,0))+IF(AH3="y",1,0)+IF(AI3="y",1,0)+IF(AJ3="y",1,0)+IF(AK3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM3" s="24"/>
       <c r="AN3" s="25"/>
-      <c r="AO3" s="26"/>
-      <c r="AP3" s="27"/>
-      <c r="AQ3" s="28"/>
-      <c r="AR3" s="29"/>
+      <c r="AO3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AS3" s="72">
         <f>IFERROR((VLOOKUP(AM3,Scoring!$A:$B,2,0))+IF(AO3="y",1,0)+IF(AP3="y",1,0)+IF(AQ3="y",1,0)+IF(AR3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT3" s="24"/>
       <c r="AU3" s="25"/>
-      <c r="AV3" s="26"/>
-      <c r="AW3" s="27"/>
-      <c r="AX3" s="28"/>
-      <c r="AY3" s="29"/>
+      <c r="AV3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ3" s="72">
         <f>IFERROR((VLOOKUP(AT3,Scoring!$A:$B,2,0))+IF(AV3="y",1,0)+IF(AW3="y",1,0)+IF(AX3="y",1,0)+IF(AY3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA3" s="24"/>
       <c r="BB3" s="25"/>
-      <c r="BC3" s="26"/>
-      <c r="BD3" s="27"/>
-      <c r="BE3" s="28"/>
-      <c r="BF3" s="29"/>
+      <c r="BC3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BG3" s="72">
         <f>IFERROR((VLOOKUP(BA3,Scoring!$A:$B,2,0))+IF(BC3="y",1,0)+IF(BD3="y",1,0)+IF(BE3="y",1,0)+IF(BF3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH3" s="24"/>
       <c r="BI3" s="25"/>
-      <c r="BJ3" s="26"/>
-      <c r="BK3" s="27"/>
-      <c r="BL3" s="28"/>
-      <c r="BM3" s="29"/>
+      <c r="BJ3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BN3" s="72">
         <f>IFERROR((VLOOKUP(BH3,Scoring!$A:$B,2,0))+IF(BJ3="y",1,0)+IF(BK3="y",1,0)+IF(BL3="y",1,0)+IF(BM3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO3" s="24"/>
       <c r="BP3" s="25"/>
-      <c r="BQ3" s="26"/>
-      <c r="BR3" s="27"/>
-      <c r="BS3" s="28"/>
-      <c r="BT3" s="29"/>
+      <c r="BQ3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BU3" s="72">
         <f>IFERROR((VLOOKUP(BO3,Scoring!$A:$B,2,0))+IF(BQ3="y",1,0)+IF(BR3="y",1,0)+IF(BS3="y",1,0)+IF(BT3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV3" s="24"/>
       <c r="BW3" s="25"/>
-      <c r="BX3" s="26"/>
-      <c r="BY3" s="27"/>
-      <c r="BZ3" s="28"/>
-      <c r="CA3" s="29"/>
+      <c r="BX3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CB3" s="72">
         <f>IFERROR((VLOOKUP(BV3,Scoring!$A:$B,2,0))+IF(BX3="y",1,0)+IF(BY3="y",1,0)+IF(BZ3="y",1,0)+IF(CA3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC3" s="24"/>
       <c r="CD3" s="25"/>
-      <c r="CE3" s="26"/>
-      <c r="CF3" s="27"/>
-      <c r="CG3" s="28"/>
-      <c r="CH3" s="29"/>
+      <c r="CE3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CI3" s="72">
         <f>IFERROR((VLOOKUP(CC3,Scoring!$A:$B,2,0))+IF(CE3="y",1,0)+IF(CF3="y",1,0)+IF(CG3="y",1,0)+IF(CH3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ3" s="24"/>
       <c r="CK3" s="25"/>
-      <c r="CL3" s="26"/>
-      <c r="CM3" s="27"/>
-      <c r="CN3" s="28"/>
-      <c r="CO3" s="29"/>
+      <c r="CL3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CP3" s="72">
         <f>IFERROR((VLOOKUP(CJ3,Scoring!$A:$B,2,0))+IF(CL3="y",1,0)+IF(CM3="y",1,0)+IF(CN3="y",1,0)+IF(CO3="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ3" s="24"/>
       <c r="CR3" s="25"/>
-      <c r="CS3" s="26"/>
-      <c r="CT3" s="27"/>
-      <c r="CU3" s="28"/>
-      <c r="CV3" s="29"/>
+      <c r="CS3" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT3" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU3" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV3" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CW3" s="72">
         <f>IFERROR((VLOOKUP(CQ3,Scoring!$A:$B,2,0))+IF(CS3="y",1,0)+IF(CT3="y",1,0)+IF(CU3="y",1,0)+IF(CV3="y",1,0),0)</f>
         <v>0</v>
@@ -3220,12 +3372,8 @@
       <c r="C4" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="36">
-        <v>3.0</v>
-      </c>
-      <c r="E4" s="37">
-        <v>14.0</v>
-      </c>
+      <c r="D4" s="36"/>
+      <c r="E4" s="37"/>
       <c r="F4" s="38" t="s">
         <v>128</v>
       </c>
@@ -3233,21 +3381,17 @@
         <v>128</v>
       </c>
       <c r="H4" s="40" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I4" s="41" t="s">
         <v>128</v>
       </c>
       <c r="J4" s="71">
         <f>IFERROR((VLOOKUP(D4,Scoring!$A:$B,2,0))+IF(F4="y",1,0)+IF(G4="y",1,0)+IF(H4="y",1,0)+IF(I4="y",1,0),0)</f>
-        <v>16</v>
-      </c>
-      <c r="K4" s="36">
-        <v>6.0</v>
-      </c>
-      <c r="L4" s="37">
-        <v>3.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K4" s="36"/>
+      <c r="L4" s="37"/>
       <c r="M4" s="38" t="s">
         <v>128</v>
       </c>
@@ -3262,14 +3406,10 @@
       </c>
       <c r="Q4" s="71">
         <f>IFERROR((VLOOKUP(K4,Scoring!$A:$B,2,0))+IF(M4="y",1,0)+IF(N4="y",1,0)+IF(O4="y",1,0)+IF(P4="y",1,0),0)</f>
-        <v>8</v>
-      </c>
-      <c r="R4" s="36">
-        <v>12.0</v>
-      </c>
-      <c r="S4" s="37">
-        <v>12.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R4" s="36"/>
+      <c r="S4" s="37"/>
       <c r="T4" s="38" t="s">
         <v>128</v>
       </c>
@@ -3284,114 +3424,202 @@
       </c>
       <c r="X4" s="71">
         <f>IFERROR((VLOOKUP(R4,Scoring!$A:$B,2,0))+IF(T4="y",1,0)+IF(U4="y",1,0)+IF(V4="y",1,0)+IF(W4="y",1,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="36"/>
       <c r="Z4" s="37"/>
-      <c r="AA4" s="38"/>
-      <c r="AB4" s="39"/>
-      <c r="AC4" s="40"/>
-      <c r="AD4" s="41"/>
+      <c r="AA4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AE4" s="71">
         <f>IFERROR((VLOOKUP(Y4,Scoring!$A:$B,2,0))+IF(AA4="y",1,0)+IF(AB4="y",1,0)+IF(AC4="y",1,0)+IF(AD4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF4" s="36"/>
       <c r="AG4" s="37"/>
-      <c r="AH4" s="38"/>
-      <c r="AI4" s="39"/>
-      <c r="AJ4" s="40"/>
-      <c r="AK4" s="41"/>
+      <c r="AH4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AL4" s="71">
         <f>IFERROR((VLOOKUP(AF4,Scoring!$A:$B,2,0))+IF(AH4="y",1,0)+IF(AI4="y",1,0)+IF(AJ4="y",1,0)+IF(AK4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM4" s="36"/>
       <c r="AN4" s="37"/>
-      <c r="AO4" s="38"/>
-      <c r="AP4" s="39"/>
-      <c r="AQ4" s="40"/>
-      <c r="AR4" s="41"/>
+      <c r="AO4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AS4" s="71">
         <f>IFERROR((VLOOKUP(AM4,Scoring!$A:$B,2,0))+IF(AO4="y",1,0)+IF(AP4="y",1,0)+IF(AQ4="y",1,0)+IF(AR4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT4" s="36"/>
       <c r="AU4" s="37"/>
-      <c r="AV4" s="38"/>
-      <c r="AW4" s="39"/>
-      <c r="AX4" s="40"/>
-      <c r="AY4" s="41"/>
+      <c r="AV4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ4" s="71">
         <f>IFERROR((VLOOKUP(AT4,Scoring!$A:$B,2,0))+IF(AV4="y",1,0)+IF(AW4="y",1,0)+IF(AX4="y",1,0)+IF(AY4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA4" s="36"/>
       <c r="BB4" s="37"/>
-      <c r="BC4" s="38"/>
-      <c r="BD4" s="39"/>
-      <c r="BE4" s="40"/>
-      <c r="BF4" s="41"/>
+      <c r="BC4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BG4" s="71">
         <f>IFERROR((VLOOKUP(BA4,Scoring!$A:$B,2,0))+IF(BC4="y",1,0)+IF(BD4="y",1,0)+IF(BE4="y",1,0)+IF(BF4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH4" s="36"/>
       <c r="BI4" s="37"/>
-      <c r="BJ4" s="38"/>
-      <c r="BK4" s="39"/>
-      <c r="BL4" s="40"/>
-      <c r="BM4" s="41"/>
+      <c r="BJ4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BN4" s="71">
         <f>IFERROR((VLOOKUP(BH4,Scoring!$A:$B,2,0))+IF(BJ4="y",1,0)+IF(BK4="y",1,0)+IF(BL4="y",1,0)+IF(BM4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO4" s="36"/>
       <c r="BP4" s="37"/>
-      <c r="BQ4" s="38"/>
-      <c r="BR4" s="39"/>
-      <c r="BS4" s="40"/>
-      <c r="BT4" s="41"/>
+      <c r="BQ4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BU4" s="71">
         <f>IFERROR((VLOOKUP(BO4,Scoring!$A:$B,2,0))+IF(BQ4="y",1,0)+IF(BR4="y",1,0)+IF(BS4="y",1,0)+IF(BT4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV4" s="36"/>
       <c r="BW4" s="37"/>
-      <c r="BX4" s="38"/>
-      <c r="BY4" s="39"/>
-      <c r="BZ4" s="40"/>
-      <c r="CA4" s="41"/>
+      <c r="BX4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CB4" s="71">
         <f>IFERROR((VLOOKUP(BV4,Scoring!$A:$B,2,0))+IF(BX4="y",1,0)+IF(BY4="y",1,0)+IF(BZ4="y",1,0)+IF(CA4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC4" s="36"/>
       <c r="CD4" s="37"/>
-      <c r="CE4" s="38"/>
-      <c r="CF4" s="39"/>
-      <c r="CG4" s="40"/>
-      <c r="CH4" s="41"/>
+      <c r="CE4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CI4" s="71">
         <f>IFERROR((VLOOKUP(CC4,Scoring!$A:$B,2,0))+IF(CE4="y",1,0)+IF(CF4="y",1,0)+IF(CG4="y",1,0)+IF(CH4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ4" s="36"/>
       <c r="CK4" s="37"/>
-      <c r="CL4" s="38"/>
-      <c r="CM4" s="39"/>
-      <c r="CN4" s="40"/>
-      <c r="CO4" s="41"/>
+      <c r="CL4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CP4" s="71">
         <f>IFERROR((VLOOKUP(CJ4,Scoring!$A:$B,2,0))+IF(CL4="y",1,0)+IF(CM4="y",1,0)+IF(CN4="y",1,0)+IF(CO4="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ4" s="36"/>
       <c r="CR4" s="37"/>
-      <c r="CS4" s="38"/>
-      <c r="CT4" s="39"/>
-      <c r="CU4" s="40"/>
-      <c r="CV4" s="41"/>
+      <c r="CS4" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT4" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU4" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV4" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CW4" s="71">
         <f>IFERROR((VLOOKUP(CQ4,Scoring!$A:$B,2,0))+IF(CS4="y",1,0)+IF(CT4="y",1,0)+IF(CU4="y",1,0)+IF(CV4="y",1,0),0)</f>
         <v>0</v>
@@ -3410,12 +3638,8 @@
       <c r="C5" s="47" t="s">
         <v>395</v>
       </c>
-      <c r="D5" s="48">
-        <v>4.0</v>
-      </c>
-      <c r="E5" s="49">
-        <v>13.0</v>
-      </c>
+      <c r="D5" s="48"/>
+      <c r="E5" s="49"/>
       <c r="F5" s="50" t="s">
         <v>128</v>
       </c>
@@ -3426,18 +3650,14 @@
         <v>128</v>
       </c>
       <c r="I5" s="53" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J5" s="72">
         <f>IFERROR((VLOOKUP(D5,Scoring!$A:$B,2,0))+IF(F5="y",1,0)+IF(G5="y",1,0)+IF(H5="y",1,0)+IF(I5="y",1,0),0)</f>
-        <v>13</v>
-      </c>
-      <c r="K5" s="48">
-        <v>8.0</v>
-      </c>
-      <c r="L5" s="49">
-        <v>4.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K5" s="48"/>
+      <c r="L5" s="49"/>
       <c r="M5" s="50" t="s">
         <v>128</v>
       </c>
@@ -3452,14 +3672,10 @@
       </c>
       <c r="Q5" s="72">
         <f>IFERROR((VLOOKUP(K5,Scoring!$A:$B,2,0))+IF(M5="y",1,0)+IF(N5="y",1,0)+IF(O5="y",1,0)+IF(P5="y",1,0),0)</f>
-        <v>4</v>
-      </c>
-      <c r="R5" s="48">
-        <v>10.0</v>
-      </c>
-      <c r="S5" s="49">
-        <v>10.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R5" s="48"/>
+      <c r="S5" s="49"/>
       <c r="T5" s="50" t="s">
         <v>128</v>
       </c>
@@ -3474,114 +3690,202 @@
       </c>
       <c r="X5" s="72">
         <f>IFERROR((VLOOKUP(R5,Scoring!$A:$B,2,0))+IF(T5="y",1,0)+IF(U5="y",1,0)+IF(V5="y",1,0)+IF(W5="y",1,0),0)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="48"/>
       <c r="Z5" s="49"/>
-      <c r="AA5" s="50"/>
-      <c r="AB5" s="51"/>
-      <c r="AC5" s="52"/>
-      <c r="AD5" s="53"/>
+      <c r="AA5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AE5" s="72">
         <f>IFERROR((VLOOKUP(Y5,Scoring!$A:$B,2,0))+IF(AA5="y",1,0)+IF(AB5="y",1,0)+IF(AC5="y",1,0)+IF(AD5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF5" s="48"/>
       <c r="AG5" s="49"/>
-      <c r="AH5" s="50"/>
-      <c r="AI5" s="51"/>
-      <c r="AJ5" s="52"/>
-      <c r="AK5" s="53"/>
+      <c r="AH5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AL5" s="72">
         <f>IFERROR((VLOOKUP(AF5,Scoring!$A:$B,2,0))+IF(AH5="y",1,0)+IF(AI5="y",1,0)+IF(AJ5="y",1,0)+IF(AK5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM5" s="48"/>
       <c r="AN5" s="49"/>
-      <c r="AO5" s="50"/>
-      <c r="AP5" s="51"/>
-      <c r="AQ5" s="52"/>
-      <c r="AR5" s="53"/>
+      <c r="AO5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AS5" s="72">
         <f>IFERROR((VLOOKUP(AM5,Scoring!$A:$B,2,0))+IF(AO5="y",1,0)+IF(AP5="y",1,0)+IF(AQ5="y",1,0)+IF(AR5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT5" s="48"/>
       <c r="AU5" s="49"/>
-      <c r="AV5" s="50"/>
-      <c r="AW5" s="51"/>
-      <c r="AX5" s="52"/>
-      <c r="AY5" s="53"/>
+      <c r="AV5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ5" s="72">
         <f>IFERROR((VLOOKUP(AT5,Scoring!$A:$B,2,0))+IF(AV5="y",1,0)+IF(AW5="y",1,0)+IF(AX5="y",1,0)+IF(AY5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA5" s="48"/>
       <c r="BB5" s="49"/>
-      <c r="BC5" s="50"/>
-      <c r="BD5" s="51"/>
-      <c r="BE5" s="52"/>
-      <c r="BF5" s="53"/>
+      <c r="BC5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BG5" s="72">
         <f>IFERROR((VLOOKUP(BA5,Scoring!$A:$B,2,0))+IF(BC5="y",1,0)+IF(BD5="y",1,0)+IF(BE5="y",1,0)+IF(BF5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH5" s="48"/>
       <c r="BI5" s="49"/>
-      <c r="BJ5" s="50"/>
-      <c r="BK5" s="51"/>
-      <c r="BL5" s="52"/>
-      <c r="BM5" s="53"/>
+      <c r="BJ5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BN5" s="72">
         <f>IFERROR((VLOOKUP(BH5,Scoring!$A:$B,2,0))+IF(BJ5="y",1,0)+IF(BK5="y",1,0)+IF(BL5="y",1,0)+IF(BM5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO5" s="48"/>
       <c r="BP5" s="49"/>
-      <c r="BQ5" s="50"/>
-      <c r="BR5" s="51"/>
-      <c r="BS5" s="52"/>
-      <c r="BT5" s="53"/>
+      <c r="BQ5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BU5" s="72">
         <f>IFERROR((VLOOKUP(BO5,Scoring!$A:$B,2,0))+IF(BQ5="y",1,0)+IF(BR5="y",1,0)+IF(BS5="y",1,0)+IF(BT5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV5" s="48"/>
       <c r="BW5" s="49"/>
-      <c r="BX5" s="50"/>
-      <c r="BY5" s="51"/>
-      <c r="BZ5" s="52"/>
-      <c r="CA5" s="53"/>
+      <c r="BX5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CB5" s="72">
         <f>IFERROR((VLOOKUP(BV5,Scoring!$A:$B,2,0))+IF(BX5="y",1,0)+IF(BY5="y",1,0)+IF(BZ5="y",1,0)+IF(CA5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC5" s="48"/>
       <c r="CD5" s="49"/>
-      <c r="CE5" s="50"/>
-      <c r="CF5" s="51"/>
-      <c r="CG5" s="52"/>
-      <c r="CH5" s="53"/>
+      <c r="CE5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CI5" s="72">
         <f>IFERROR((VLOOKUP(CC5,Scoring!$A:$B,2,0))+IF(CE5="y",1,0)+IF(CF5="y",1,0)+IF(CG5="y",1,0)+IF(CH5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ5" s="48"/>
       <c r="CK5" s="49"/>
-      <c r="CL5" s="50"/>
-      <c r="CM5" s="51"/>
-      <c r="CN5" s="52"/>
-      <c r="CO5" s="53"/>
+      <c r="CL5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CP5" s="72">
         <f>IFERROR((VLOOKUP(CJ5,Scoring!$A:$B,2,0))+IF(CL5="y",1,0)+IF(CM5="y",1,0)+IF(CN5="y",1,0)+IF(CO5="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ5" s="48"/>
       <c r="CR5" s="49"/>
-      <c r="CS5" s="50"/>
-      <c r="CT5" s="51"/>
-      <c r="CU5" s="52"/>
-      <c r="CV5" s="53"/>
+      <c r="CS5" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT5" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU5" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV5" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CW5" s="72">
         <f>IFERROR((VLOOKUP(CQ5,Scoring!$A:$B,2,0))+IF(CS5="y",1,0)+IF(CT5="y",1,0)+IF(CU5="y",1,0)+IF(CV5="y",1,0),0)</f>
         <v>0</v>
@@ -3600,12 +3904,8 @@
       <c r="C6" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="24">
-        <v>5.0</v>
-      </c>
-      <c r="E6" s="25">
-        <v>12.0</v>
-      </c>
+      <c r="D6" s="24"/>
+      <c r="E6" s="25"/>
       <c r="F6" s="26" t="s">
         <v>128</v>
       </c>
@@ -3620,14 +3920,10 @@
       </c>
       <c r="J6" s="71">
         <f>IFERROR((VLOOKUP(D6,Scoring!$A:$B,2,0))+IF(F6="y",1,0)+IF(G6="y",1,0)+IF(H6="y",1,0)+IF(I6="y",1,0),0)</f>
-        <v>10</v>
-      </c>
-      <c r="K6" s="24">
-        <v>10.0</v>
-      </c>
-      <c r="L6" s="25">
-        <v>5.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K6" s="24"/>
+      <c r="L6" s="25"/>
       <c r="M6" s="26" t="s">
         <v>128</v>
       </c>
@@ -3642,14 +3938,10 @@
       </c>
       <c r="Q6" s="71">
         <f>IFERROR((VLOOKUP(K6,Scoring!$A:$B,2,0))+IF(M6="y",1,0)+IF(N6="y",1,0)+IF(O6="y",1,0)+IF(P6="y",1,0),0)</f>
-        <v>2</v>
-      </c>
-      <c r="R6" s="24">
-        <v>8.0</v>
-      </c>
-      <c r="S6" s="25">
-        <v>8.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R6" s="24"/>
+      <c r="S6" s="25"/>
       <c r="T6" s="26" t="s">
         <v>128</v>
       </c>
@@ -3664,114 +3956,202 @@
       </c>
       <c r="X6" s="71">
         <f>IFERROR((VLOOKUP(R6,Scoring!$A:$B,2,0))+IF(T6="y",1,0)+IF(U6="y",1,0)+IF(V6="y",1,0)+IF(W6="y",1,0),0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Y6" s="24"/>
       <c r="Z6" s="25"/>
-      <c r="AA6" s="26"/>
-      <c r="AB6" s="27"/>
-      <c r="AC6" s="28"/>
-      <c r="AD6" s="29"/>
+      <c r="AA6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AE6" s="71">
         <f>IFERROR((VLOOKUP(Y6,Scoring!$A:$B,2,0))+IF(AA6="y",1,0)+IF(AB6="y",1,0)+IF(AC6="y",1,0)+IF(AD6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF6" s="24"/>
       <c r="AG6" s="25"/>
-      <c r="AH6" s="26"/>
-      <c r="AI6" s="27"/>
-      <c r="AJ6" s="28"/>
-      <c r="AK6" s="29"/>
+      <c r="AH6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AL6" s="71">
         <f>IFERROR((VLOOKUP(AF6,Scoring!$A:$B,2,0))+IF(AH6="y",1,0)+IF(AI6="y",1,0)+IF(AJ6="y",1,0)+IF(AK6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM6" s="24"/>
       <c r="AN6" s="25"/>
-      <c r="AO6" s="26"/>
-      <c r="AP6" s="27"/>
-      <c r="AQ6" s="28"/>
-      <c r="AR6" s="29"/>
+      <c r="AO6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AS6" s="71">
         <f>IFERROR((VLOOKUP(AM6,Scoring!$A:$B,2,0))+IF(AO6="y",1,0)+IF(AP6="y",1,0)+IF(AQ6="y",1,0)+IF(AR6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT6" s="24"/>
       <c r="AU6" s="25"/>
-      <c r="AV6" s="26"/>
-      <c r="AW6" s="27"/>
-      <c r="AX6" s="28"/>
-      <c r="AY6" s="29"/>
+      <c r="AV6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ6" s="71">
         <f>IFERROR((VLOOKUP(AT6,Scoring!$A:$B,2,0))+IF(AV6="y",1,0)+IF(AW6="y",1,0)+IF(AX6="y",1,0)+IF(AY6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA6" s="24"/>
       <c r="BB6" s="25"/>
-      <c r="BC6" s="26"/>
-      <c r="BD6" s="27"/>
-      <c r="BE6" s="28"/>
-      <c r="BF6" s="29"/>
+      <c r="BC6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BG6" s="71">
         <f>IFERROR((VLOOKUP(BA6,Scoring!$A:$B,2,0))+IF(BC6="y",1,0)+IF(BD6="y",1,0)+IF(BE6="y",1,0)+IF(BF6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH6" s="24"/>
       <c r="BI6" s="25"/>
-      <c r="BJ6" s="26"/>
-      <c r="BK6" s="27"/>
-      <c r="BL6" s="28"/>
-      <c r="BM6" s="29"/>
+      <c r="BJ6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BN6" s="71">
         <f>IFERROR((VLOOKUP(BH6,Scoring!$A:$B,2,0))+IF(BJ6="y",1,0)+IF(BK6="y",1,0)+IF(BL6="y",1,0)+IF(BM6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO6" s="24"/>
       <c r="BP6" s="25"/>
-      <c r="BQ6" s="26"/>
-      <c r="BR6" s="27"/>
-      <c r="BS6" s="28"/>
-      <c r="BT6" s="29"/>
+      <c r="BQ6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BU6" s="71">
         <f>IFERROR((VLOOKUP(BO6,Scoring!$A:$B,2,0))+IF(BQ6="y",1,0)+IF(BR6="y",1,0)+IF(BS6="y",1,0)+IF(BT6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV6" s="24"/>
       <c r="BW6" s="25"/>
-      <c r="BX6" s="26"/>
-      <c r="BY6" s="27"/>
-      <c r="BZ6" s="28"/>
-      <c r="CA6" s="29"/>
+      <c r="BX6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CB6" s="71">
         <f>IFERROR((VLOOKUP(BV6,Scoring!$A:$B,2,0))+IF(BX6="y",1,0)+IF(BY6="y",1,0)+IF(BZ6="y",1,0)+IF(CA6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC6" s="24"/>
       <c r="CD6" s="25"/>
-      <c r="CE6" s="26"/>
-      <c r="CF6" s="27"/>
-      <c r="CG6" s="28"/>
-      <c r="CH6" s="29"/>
+      <c r="CE6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CI6" s="71">
         <f>IFERROR((VLOOKUP(CC6,Scoring!$A:$B,2,0))+IF(CE6="y",1,0)+IF(CF6="y",1,0)+IF(CG6="y",1,0)+IF(CH6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ6" s="24"/>
       <c r="CK6" s="25"/>
-      <c r="CL6" s="26"/>
-      <c r="CM6" s="27"/>
-      <c r="CN6" s="28"/>
-      <c r="CO6" s="29"/>
+      <c r="CL6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CP6" s="71">
         <f>IFERROR((VLOOKUP(CJ6,Scoring!$A:$B,2,0))+IF(CL6="y",1,0)+IF(CM6="y",1,0)+IF(CN6="y",1,0)+IF(CO6="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ6" s="24"/>
       <c r="CR6" s="25"/>
-      <c r="CS6" s="26"/>
-      <c r="CT6" s="27"/>
-      <c r="CU6" s="28"/>
-      <c r="CV6" s="29"/>
+      <c r="CS6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT6" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU6" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV6" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CW6" s="71">
         <f>IFERROR((VLOOKUP(CQ6,Scoring!$A:$B,2,0))+IF(CS6="y",1,0)+IF(CT6="y",1,0)+IF(CU6="y",1,0)+IF(CV6="y",1,0),0)</f>
         <v>0</v>
@@ -3790,12 +4170,8 @@
       <c r="C7" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="24">
-        <v>6.0</v>
-      </c>
-      <c r="E7" s="25">
-        <v>11.0</v>
-      </c>
+      <c r="D7" s="24"/>
+      <c r="E7" s="25"/>
       <c r="F7" s="26" t="s">
         <v>128</v>
       </c>
@@ -3810,14 +4186,10 @@
       </c>
       <c r="J7" s="72">
         <f>IFERROR((VLOOKUP(D7,Scoring!$A:$B,2,0))+IF(F7="y",1,0)+IF(G7="y",1,0)+IF(H7="y",1,0)+IF(I7="y",1,0),0)</f>
-        <v>8</v>
-      </c>
-      <c r="K7" s="24">
-        <v>12.0</v>
-      </c>
-      <c r="L7" s="25">
-        <v>6.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K7" s="24"/>
+      <c r="L7" s="25"/>
       <c r="M7" s="26" t="s">
         <v>128</v>
       </c>
@@ -3832,14 +4204,10 @@
       </c>
       <c r="Q7" s="72">
         <f>IFERROR((VLOOKUP(K7,Scoring!$A:$B,2,0))+IF(M7="y",1,0)+IF(N7="y",1,0)+IF(O7="y",1,0)+IF(P7="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="R7" s="24">
-        <v>6.0</v>
-      </c>
-      <c r="S7" s="25">
-        <v>6.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R7" s="24"/>
+      <c r="S7" s="25"/>
       <c r="T7" s="26" t="s">
         <v>128</v>
       </c>
@@ -3854,114 +4222,202 @@
       </c>
       <c r="X7" s="72">
         <f>IFERROR((VLOOKUP(R7,Scoring!$A:$B,2,0))+IF(T7="y",1,0)+IF(U7="y",1,0)+IF(V7="y",1,0)+IF(W7="y",1,0),0)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="24"/>
       <c r="Z7" s="25"/>
-      <c r="AA7" s="26"/>
-      <c r="AB7" s="27"/>
-      <c r="AC7" s="28"/>
-      <c r="AD7" s="29"/>
+      <c r="AA7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AE7" s="72">
         <f>IFERROR((VLOOKUP(Y7,Scoring!$A:$B,2,0))+IF(AA7="y",1,0)+IF(AB7="y",1,0)+IF(AC7="y",1,0)+IF(AD7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF7" s="24"/>
       <c r="AG7" s="25"/>
-      <c r="AH7" s="26"/>
-      <c r="AI7" s="27"/>
-      <c r="AJ7" s="28"/>
-      <c r="AK7" s="29"/>
+      <c r="AH7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AL7" s="72">
         <f>IFERROR((VLOOKUP(AF7,Scoring!$A:$B,2,0))+IF(AH7="y",1,0)+IF(AI7="y",1,0)+IF(AJ7="y",1,0)+IF(AK7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM7" s="24"/>
       <c r="AN7" s="25"/>
-      <c r="AO7" s="26"/>
-      <c r="AP7" s="27"/>
-      <c r="AQ7" s="28"/>
-      <c r="AR7" s="29"/>
+      <c r="AO7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AS7" s="72">
         <f>IFERROR((VLOOKUP(AM7,Scoring!$A:$B,2,0))+IF(AO7="y",1,0)+IF(AP7="y",1,0)+IF(AQ7="y",1,0)+IF(AR7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT7" s="24"/>
       <c r="AU7" s="25"/>
-      <c r="AV7" s="26"/>
-      <c r="AW7" s="27"/>
-      <c r="AX7" s="28"/>
-      <c r="AY7" s="29"/>
+      <c r="AV7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ7" s="72">
         <f>IFERROR((VLOOKUP(AT7,Scoring!$A:$B,2,0))+IF(AV7="y",1,0)+IF(AW7="y",1,0)+IF(AX7="y",1,0)+IF(AY7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA7" s="24"/>
       <c r="BB7" s="25"/>
-      <c r="BC7" s="26"/>
-      <c r="BD7" s="27"/>
-      <c r="BE7" s="28"/>
-      <c r="BF7" s="29"/>
+      <c r="BC7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BG7" s="72">
         <f>IFERROR((VLOOKUP(BA7,Scoring!$A:$B,2,0))+IF(BC7="y",1,0)+IF(BD7="y",1,0)+IF(BE7="y",1,0)+IF(BF7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH7" s="24"/>
       <c r="BI7" s="25"/>
-      <c r="BJ7" s="26"/>
-      <c r="BK7" s="27"/>
-      <c r="BL7" s="28"/>
-      <c r="BM7" s="29"/>
+      <c r="BJ7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BN7" s="72">
         <f>IFERROR((VLOOKUP(BH7,Scoring!$A:$B,2,0))+IF(BJ7="y",1,0)+IF(BK7="y",1,0)+IF(BL7="y",1,0)+IF(BM7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO7" s="24"/>
       <c r="BP7" s="25"/>
-      <c r="BQ7" s="26"/>
-      <c r="BR7" s="27"/>
-      <c r="BS7" s="28"/>
-      <c r="BT7" s="29"/>
+      <c r="BQ7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BU7" s="72">
         <f>IFERROR((VLOOKUP(BO7,Scoring!$A:$B,2,0))+IF(BQ7="y",1,0)+IF(BR7="y",1,0)+IF(BS7="y",1,0)+IF(BT7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV7" s="24"/>
       <c r="BW7" s="25"/>
-      <c r="BX7" s="26"/>
-      <c r="BY7" s="27"/>
-      <c r="BZ7" s="28"/>
-      <c r="CA7" s="29"/>
+      <c r="BX7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CB7" s="72">
         <f>IFERROR((VLOOKUP(BV7,Scoring!$A:$B,2,0))+IF(BX7="y",1,0)+IF(BY7="y",1,0)+IF(BZ7="y",1,0)+IF(CA7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC7" s="24"/>
       <c r="CD7" s="25"/>
-      <c r="CE7" s="26"/>
-      <c r="CF7" s="27"/>
-      <c r="CG7" s="28"/>
-      <c r="CH7" s="29"/>
+      <c r="CE7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CI7" s="72">
         <f>IFERROR((VLOOKUP(CC7,Scoring!$A:$B,2,0))+IF(CE7="y",1,0)+IF(CF7="y",1,0)+IF(CG7="y",1,0)+IF(CH7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ7" s="24"/>
       <c r="CK7" s="25"/>
-      <c r="CL7" s="26"/>
-      <c r="CM7" s="27"/>
-      <c r="CN7" s="28"/>
-      <c r="CO7" s="29"/>
+      <c r="CL7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CP7" s="72">
         <f>IFERROR((VLOOKUP(CJ7,Scoring!$A:$B,2,0))+IF(CL7="y",1,0)+IF(CM7="y",1,0)+IF(CN7="y",1,0)+IF(CO7="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ7" s="24"/>
       <c r="CR7" s="25"/>
-      <c r="CS7" s="26"/>
-      <c r="CT7" s="27"/>
-      <c r="CU7" s="28"/>
-      <c r="CV7" s="29"/>
+      <c r="CS7" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT7" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU7" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV7" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CW7" s="72">
         <f>IFERROR((VLOOKUP(CQ7,Scoring!$A:$B,2,0))+IF(CS7="y",1,0)+IF(CT7="y",1,0)+IF(CU7="y",1,0)+IF(CV7="y",1,0),0)</f>
         <v>0</v>
@@ -3980,12 +4436,8 @@
       <c r="C8" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="36">
-        <v>7.0</v>
-      </c>
-      <c r="E8" s="37">
-        <v>10.0</v>
-      </c>
+      <c r="D8" s="36"/>
+      <c r="E8" s="37"/>
       <c r="F8" s="38" t="s">
         <v>128</v>
       </c>
@@ -4000,14 +4452,10 @@
       </c>
       <c r="J8" s="71">
         <f>IFERROR((VLOOKUP(D8,Scoring!$A:$B,2,0))+IF(F8="y",1,0)+IF(G8="y",1,0)+IF(H8="y",1,0)+IF(I8="y",1,0),0)</f>
-        <v>6</v>
-      </c>
-      <c r="K8" s="36">
-        <v>14.0</v>
-      </c>
-      <c r="L8" s="37">
-        <v>7.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K8" s="36"/>
+      <c r="L8" s="37"/>
       <c r="M8" s="38" t="s">
         <v>128</v>
       </c>
@@ -4022,14 +4470,10 @@
       </c>
       <c r="Q8" s="71">
         <f>IFERROR((VLOOKUP(K8,Scoring!$A:$B,2,0))+IF(M8="y",1,0)+IF(N8="y",1,0)+IF(O8="y",1,0)+IF(P8="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="R8" s="36">
-        <v>4.0</v>
-      </c>
-      <c r="S8" s="37">
-        <v>4.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R8" s="36"/>
+      <c r="S8" s="37"/>
       <c r="T8" s="38" t="s">
         <v>128</v>
       </c>
@@ -4044,114 +4488,202 @@
       </c>
       <c r="X8" s="71">
         <f>IFERROR((VLOOKUP(R8,Scoring!$A:$B,2,0))+IF(T8="y",1,0)+IF(U8="y",1,0)+IF(V8="y",1,0)+IF(W8="y",1,0),0)</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y8" s="36"/>
       <c r="Z8" s="37"/>
-      <c r="AA8" s="38"/>
-      <c r="AB8" s="39"/>
-      <c r="AC8" s="40"/>
-      <c r="AD8" s="41"/>
+      <c r="AA8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AE8" s="71">
         <f>IFERROR((VLOOKUP(Y8,Scoring!$A:$B,2,0))+IF(AA8="y",1,0)+IF(AB8="y",1,0)+IF(AC8="y",1,0)+IF(AD8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF8" s="36"/>
       <c r="AG8" s="37"/>
-      <c r="AH8" s="38"/>
-      <c r="AI8" s="39"/>
-      <c r="AJ8" s="40"/>
-      <c r="AK8" s="41"/>
+      <c r="AH8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AL8" s="71">
         <f>IFERROR((VLOOKUP(AF8,Scoring!$A:$B,2,0))+IF(AH8="y",1,0)+IF(AI8="y",1,0)+IF(AJ8="y",1,0)+IF(AK8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM8" s="36"/>
       <c r="AN8" s="37"/>
-      <c r="AO8" s="38"/>
-      <c r="AP8" s="39"/>
-      <c r="AQ8" s="40"/>
-      <c r="AR8" s="41"/>
+      <c r="AO8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AS8" s="71">
         <f>IFERROR((VLOOKUP(AM8,Scoring!$A:$B,2,0))+IF(AO8="y",1,0)+IF(AP8="y",1,0)+IF(AQ8="y",1,0)+IF(AR8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT8" s="36"/>
       <c r="AU8" s="37"/>
-      <c r="AV8" s="38"/>
-      <c r="AW8" s="39"/>
-      <c r="AX8" s="40"/>
-      <c r="AY8" s="41"/>
+      <c r="AV8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ8" s="71">
         <f>IFERROR((VLOOKUP(AT8,Scoring!$A:$B,2,0))+IF(AV8="y",1,0)+IF(AW8="y",1,0)+IF(AX8="y",1,0)+IF(AY8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA8" s="36"/>
       <c r="BB8" s="37"/>
-      <c r="BC8" s="38"/>
-      <c r="BD8" s="39"/>
-      <c r="BE8" s="40"/>
-      <c r="BF8" s="41"/>
+      <c r="BC8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BG8" s="71">
         <f>IFERROR((VLOOKUP(BA8,Scoring!$A:$B,2,0))+IF(BC8="y",1,0)+IF(BD8="y",1,0)+IF(BE8="y",1,0)+IF(BF8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH8" s="36"/>
       <c r="BI8" s="37"/>
-      <c r="BJ8" s="38"/>
-      <c r="BK8" s="39"/>
-      <c r="BL8" s="40"/>
-      <c r="BM8" s="41"/>
+      <c r="BJ8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BN8" s="71">
         <f>IFERROR((VLOOKUP(BH8,Scoring!$A:$B,2,0))+IF(BJ8="y",1,0)+IF(BK8="y",1,0)+IF(BL8="y",1,0)+IF(BM8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO8" s="36"/>
       <c r="BP8" s="37"/>
-      <c r="BQ8" s="38"/>
-      <c r="BR8" s="39"/>
-      <c r="BS8" s="40"/>
-      <c r="BT8" s="41"/>
+      <c r="BQ8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BU8" s="71">
         <f>IFERROR((VLOOKUP(BO8,Scoring!$A:$B,2,0))+IF(BQ8="y",1,0)+IF(BR8="y",1,0)+IF(BS8="y",1,0)+IF(BT8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV8" s="36"/>
       <c r="BW8" s="37"/>
-      <c r="BX8" s="38"/>
-      <c r="BY8" s="39"/>
-      <c r="BZ8" s="40"/>
-      <c r="CA8" s="41"/>
+      <c r="BX8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CB8" s="71">
         <f>IFERROR((VLOOKUP(BV8,Scoring!$A:$B,2,0))+IF(BX8="y",1,0)+IF(BY8="y",1,0)+IF(BZ8="y",1,0)+IF(CA8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC8" s="36"/>
       <c r="CD8" s="37"/>
-      <c r="CE8" s="38"/>
-      <c r="CF8" s="39"/>
-      <c r="CG8" s="40"/>
-      <c r="CH8" s="41"/>
+      <c r="CE8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CI8" s="71">
         <f>IFERROR((VLOOKUP(CC8,Scoring!$A:$B,2,0))+IF(CE8="y",1,0)+IF(CF8="y",1,0)+IF(CG8="y",1,0)+IF(CH8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ8" s="36"/>
       <c r="CK8" s="37"/>
-      <c r="CL8" s="38"/>
-      <c r="CM8" s="39"/>
-      <c r="CN8" s="40"/>
-      <c r="CO8" s="41"/>
+      <c r="CL8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CP8" s="71">
         <f>IFERROR((VLOOKUP(CJ8,Scoring!$A:$B,2,0))+IF(CL8="y",1,0)+IF(CM8="y",1,0)+IF(CN8="y",1,0)+IF(CO8="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ8" s="36"/>
       <c r="CR8" s="37"/>
-      <c r="CS8" s="38"/>
-      <c r="CT8" s="39"/>
-      <c r="CU8" s="40"/>
-      <c r="CV8" s="41"/>
+      <c r="CS8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT8" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU8" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV8" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CW8" s="71">
         <f>IFERROR((VLOOKUP(CQ8,Scoring!$A:$B,2,0))+IF(CS8="y",1,0)+IF(CT8="y",1,0)+IF(CU8="y",1,0)+IF(CV8="y",1,0),0)</f>
         <v>0</v>
@@ -4170,12 +4702,8 @@
       <c r="C9" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="48">
-        <v>8.0</v>
-      </c>
-      <c r="E9" s="49">
-        <v>9.0</v>
-      </c>
+      <c r="D9" s="48"/>
+      <c r="E9" s="49"/>
       <c r="F9" s="50" t="s">
         <v>128</v>
       </c>
@@ -4190,14 +4718,10 @@
       </c>
       <c r="J9" s="72">
         <f>IFERROR((VLOOKUP(D9,Scoring!$A:$B,2,0))+IF(F9="y",1,0)+IF(G9="y",1,0)+IF(H9="y",1,0)+IF(I9="y",1,0),0)</f>
-        <v>4</v>
-      </c>
-      <c r="K9" s="48">
-        <v>16.0</v>
-      </c>
-      <c r="L9" s="49">
-        <v>8.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K9" s="48"/>
+      <c r="L9" s="49"/>
       <c r="M9" s="50" t="s">
         <v>128</v>
       </c>
@@ -4212,14 +4736,10 @@
       </c>
       <c r="Q9" s="72">
         <f>IFERROR((VLOOKUP(K9,Scoring!$A:$B,2,0))+IF(M9="y",1,0)+IF(N9="y",1,0)+IF(O9="y",1,0)+IF(P9="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="R9" s="48">
-        <v>2.0</v>
-      </c>
-      <c r="S9" s="49">
-        <v>2.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R9" s="48"/>
+      <c r="S9" s="49"/>
       <c r="T9" s="50" t="s">
         <v>128</v>
       </c>
@@ -4234,114 +4754,202 @@
       </c>
       <c r="X9" s="72">
         <f>IFERROR((VLOOKUP(R9,Scoring!$A:$B,2,0))+IF(T9="y",1,0)+IF(U9="y",1,0)+IF(V9="y",1,0)+IF(W9="y",1,0),0)</f>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="Y9" s="48"/>
       <c r="Z9" s="49"/>
-      <c r="AA9" s="50"/>
-      <c r="AB9" s="51"/>
-      <c r="AC9" s="52"/>
-      <c r="AD9" s="53"/>
+      <c r="AA9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AE9" s="72">
         <f>IFERROR((VLOOKUP(Y9,Scoring!$A:$B,2,0))+IF(AA9="y",1,0)+IF(AB9="y",1,0)+IF(AC9="y",1,0)+IF(AD9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF9" s="48"/>
       <c r="AG9" s="49"/>
-      <c r="AH9" s="50"/>
-      <c r="AI9" s="51"/>
-      <c r="AJ9" s="52"/>
-      <c r="AK9" s="53"/>
+      <c r="AH9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AL9" s="72">
         <f>IFERROR((VLOOKUP(AF9,Scoring!$A:$B,2,0))+IF(AH9="y",1,0)+IF(AI9="y",1,0)+IF(AJ9="y",1,0)+IF(AK9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM9" s="48"/>
       <c r="AN9" s="49"/>
-      <c r="AO9" s="50"/>
-      <c r="AP9" s="51"/>
-      <c r="AQ9" s="52"/>
-      <c r="AR9" s="53"/>
+      <c r="AO9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AS9" s="72">
         <f>IFERROR((VLOOKUP(AM9,Scoring!$A:$B,2,0))+IF(AO9="y",1,0)+IF(AP9="y",1,0)+IF(AQ9="y",1,0)+IF(AR9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT9" s="48"/>
       <c r="AU9" s="49"/>
-      <c r="AV9" s="50"/>
-      <c r="AW9" s="51"/>
-      <c r="AX9" s="52"/>
-      <c r="AY9" s="53"/>
+      <c r="AV9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ9" s="72">
         <f>IFERROR((VLOOKUP(AT9,Scoring!$A:$B,2,0))+IF(AV9="y",1,0)+IF(AW9="y",1,0)+IF(AX9="y",1,0)+IF(AY9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA9" s="48"/>
       <c r="BB9" s="49"/>
-      <c r="BC9" s="50"/>
-      <c r="BD9" s="51"/>
-      <c r="BE9" s="52"/>
-      <c r="BF9" s="53"/>
+      <c r="BC9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BG9" s="72">
         <f>IFERROR((VLOOKUP(BA9,Scoring!$A:$B,2,0))+IF(BC9="y",1,0)+IF(BD9="y",1,0)+IF(BE9="y",1,0)+IF(BF9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH9" s="48"/>
       <c r="BI9" s="49"/>
-      <c r="BJ9" s="50"/>
-      <c r="BK9" s="51"/>
-      <c r="BL9" s="52"/>
-      <c r="BM9" s="53"/>
+      <c r="BJ9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BN9" s="72">
         <f>IFERROR((VLOOKUP(BH9,Scoring!$A:$B,2,0))+IF(BJ9="y",1,0)+IF(BK9="y",1,0)+IF(BL9="y",1,0)+IF(BM9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO9" s="48"/>
       <c r="BP9" s="49"/>
-      <c r="BQ9" s="50"/>
-      <c r="BR9" s="51"/>
-      <c r="BS9" s="52"/>
-      <c r="BT9" s="53"/>
+      <c r="BQ9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BU9" s="72">
         <f>IFERROR((VLOOKUP(BO9,Scoring!$A:$B,2,0))+IF(BQ9="y",1,0)+IF(BR9="y",1,0)+IF(BS9="y",1,0)+IF(BT9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV9" s="48"/>
       <c r="BW9" s="49"/>
-      <c r="BX9" s="50"/>
-      <c r="BY9" s="51"/>
-      <c r="BZ9" s="52"/>
-      <c r="CA9" s="53"/>
+      <c r="BX9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CB9" s="72">
         <f>IFERROR((VLOOKUP(BV9,Scoring!$A:$B,2,0))+IF(BX9="y",1,0)+IF(BY9="y",1,0)+IF(BZ9="y",1,0)+IF(CA9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC9" s="48"/>
       <c r="CD9" s="49"/>
-      <c r="CE9" s="50"/>
-      <c r="CF9" s="51"/>
-      <c r="CG9" s="52"/>
-      <c r="CH9" s="53"/>
+      <c r="CE9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CI9" s="72">
         <f>IFERROR((VLOOKUP(CC9,Scoring!$A:$B,2,0))+IF(CE9="y",1,0)+IF(CF9="y",1,0)+IF(CG9="y",1,0)+IF(CH9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ9" s="48"/>
       <c r="CK9" s="49"/>
-      <c r="CL9" s="50"/>
-      <c r="CM9" s="51"/>
-      <c r="CN9" s="52"/>
-      <c r="CO9" s="53"/>
+      <c r="CL9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CP9" s="72">
         <f>IFERROR((VLOOKUP(CJ9,Scoring!$A:$B,2,0))+IF(CL9="y",1,0)+IF(CM9="y",1,0)+IF(CN9="y",1,0)+IF(CO9="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ9" s="48"/>
       <c r="CR9" s="49"/>
-      <c r="CS9" s="50"/>
-      <c r="CT9" s="51"/>
-      <c r="CU9" s="52"/>
-      <c r="CV9" s="53"/>
+      <c r="CS9" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT9" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU9" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV9" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CW9" s="72">
         <f>IFERROR((VLOOKUP(CQ9,Scoring!$A:$B,2,0))+IF(CS9="y",1,0)+IF(CT9="y",1,0)+IF(CU9="y",1,0)+IF(CV9="y",1,0),0)</f>
         <v>0</v>
@@ -4360,12 +4968,8 @@
       <c r="C10" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="24">
-        <v>9.0</v>
-      </c>
-      <c r="E10" s="25">
-        <v>8.0</v>
-      </c>
+      <c r="D10" s="24"/>
+      <c r="E10" s="25"/>
       <c r="F10" s="26" t="s">
         <v>128</v>
       </c>
@@ -4380,14 +4984,10 @@
       </c>
       <c r="J10" s="71">
         <f>IFERROR((VLOOKUP(D10,Scoring!$A:$B,2,0))+IF(F10="y",1,0)+IF(G10="y",1,0)+IF(H10="y",1,0)+IF(I10="y",1,0),0)</f>
-        <v>3</v>
-      </c>
-      <c r="K10" s="24">
-        <v>1.0</v>
-      </c>
-      <c r="L10" s="25">
-        <v>9.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K10" s="24"/>
+      <c r="L10" s="25"/>
       <c r="M10" s="26" t="s">
         <v>128</v>
       </c>
@@ -4402,14 +5002,10 @@
       </c>
       <c r="Q10" s="71">
         <f>IFERROR((VLOOKUP(K10,Scoring!$A:$B,2,0))+IF(M10="y",1,0)+IF(N10="y",1,0)+IF(O10="y",1,0)+IF(P10="y",1,0),0)</f>
-        <v>25</v>
-      </c>
-      <c r="R10" s="24">
-        <v>15.0</v>
-      </c>
-      <c r="S10" s="25">
-        <v>1.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R10" s="24"/>
+      <c r="S10" s="25"/>
       <c r="T10" s="26" t="s">
         <v>128</v>
       </c>
@@ -4424,114 +5020,202 @@
       </c>
       <c r="X10" s="71">
         <f>IFERROR((VLOOKUP(R10,Scoring!$A:$B,2,0))+IF(T10="y",1,0)+IF(U10="y",1,0)+IF(V10="y",1,0)+IF(W10="y",1,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="24"/>
       <c r="Z10" s="25"/>
-      <c r="AA10" s="26"/>
-      <c r="AB10" s="27"/>
-      <c r="AC10" s="28"/>
-      <c r="AD10" s="29"/>
+      <c r="AA10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AE10" s="71">
         <f>IFERROR((VLOOKUP(Y10,Scoring!$A:$B,2,0))+IF(AA10="y",1,0)+IF(AB10="y",1,0)+IF(AC10="y",1,0)+IF(AD10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF10" s="24"/>
       <c r="AG10" s="25"/>
-      <c r="AH10" s="26"/>
-      <c r="AI10" s="27"/>
-      <c r="AJ10" s="28"/>
-      <c r="AK10" s="29"/>
+      <c r="AH10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AL10" s="71">
         <f>IFERROR((VLOOKUP(AF10,Scoring!$A:$B,2,0))+IF(AH10="y",1,0)+IF(AI10="y",1,0)+IF(AJ10="y",1,0)+IF(AK10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM10" s="24"/>
       <c r="AN10" s="25"/>
-      <c r="AO10" s="26"/>
-      <c r="AP10" s="27"/>
-      <c r="AQ10" s="28"/>
-      <c r="AR10" s="29"/>
+      <c r="AO10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AS10" s="71">
         <f>IFERROR((VLOOKUP(AM10,Scoring!$A:$B,2,0))+IF(AO10="y",1,0)+IF(AP10="y",1,0)+IF(AQ10="y",1,0)+IF(AR10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT10" s="24"/>
       <c r="AU10" s="25"/>
-      <c r="AV10" s="26"/>
-      <c r="AW10" s="27"/>
-      <c r="AX10" s="28"/>
-      <c r="AY10" s="29"/>
+      <c r="AV10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ10" s="71">
         <f>IFERROR((VLOOKUP(AT10,Scoring!$A:$B,2,0))+IF(AV10="y",1,0)+IF(AW10="y",1,0)+IF(AX10="y",1,0)+IF(AY10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA10" s="24"/>
       <c r="BB10" s="25"/>
-      <c r="BC10" s="26"/>
-      <c r="BD10" s="27"/>
-      <c r="BE10" s="28"/>
-      <c r="BF10" s="29"/>
+      <c r="BC10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BG10" s="71">
         <f>IFERROR((VLOOKUP(BA10,Scoring!$A:$B,2,0))+IF(BC10="y",1,0)+IF(BD10="y",1,0)+IF(BE10="y",1,0)+IF(BF10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH10" s="24"/>
       <c r="BI10" s="25"/>
-      <c r="BJ10" s="26"/>
-      <c r="BK10" s="27"/>
-      <c r="BL10" s="28"/>
-      <c r="BM10" s="29"/>
+      <c r="BJ10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BN10" s="71">
         <f>IFERROR((VLOOKUP(BH10,Scoring!$A:$B,2,0))+IF(BJ10="y",1,0)+IF(BK10="y",1,0)+IF(BL10="y",1,0)+IF(BM10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO10" s="24"/>
       <c r="BP10" s="25"/>
-      <c r="BQ10" s="26"/>
-      <c r="BR10" s="27"/>
-      <c r="BS10" s="28"/>
-      <c r="BT10" s="29"/>
+      <c r="BQ10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BU10" s="71">
         <f>IFERROR((VLOOKUP(BO10,Scoring!$A:$B,2,0))+IF(BQ10="y",1,0)+IF(BR10="y",1,0)+IF(BS10="y",1,0)+IF(BT10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV10" s="24"/>
       <c r="BW10" s="25"/>
-      <c r="BX10" s="26"/>
-      <c r="BY10" s="27"/>
-      <c r="BZ10" s="28"/>
-      <c r="CA10" s="29"/>
+      <c r="BX10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CB10" s="71">
         <f>IFERROR((VLOOKUP(BV10,Scoring!$A:$B,2,0))+IF(BX10="y",1,0)+IF(BY10="y",1,0)+IF(BZ10="y",1,0)+IF(CA10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC10" s="24"/>
       <c r="CD10" s="25"/>
-      <c r="CE10" s="26"/>
-      <c r="CF10" s="27"/>
-      <c r="CG10" s="28"/>
-      <c r="CH10" s="29"/>
+      <c r="CE10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CI10" s="71">
         <f>IFERROR((VLOOKUP(CC10,Scoring!$A:$B,2,0))+IF(CE10="y",1,0)+IF(CF10="y",1,0)+IF(CG10="y",1,0)+IF(CH10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ10" s="24"/>
       <c r="CK10" s="25"/>
-      <c r="CL10" s="26"/>
-      <c r="CM10" s="27"/>
-      <c r="CN10" s="28"/>
-      <c r="CO10" s="29"/>
+      <c r="CL10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CP10" s="71">
         <f>IFERROR((VLOOKUP(CJ10,Scoring!$A:$B,2,0))+IF(CL10="y",1,0)+IF(CM10="y",1,0)+IF(CN10="y",1,0)+IF(CO10="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ10" s="24"/>
       <c r="CR10" s="25"/>
-      <c r="CS10" s="26"/>
-      <c r="CT10" s="27"/>
-      <c r="CU10" s="28"/>
-      <c r="CV10" s="29"/>
+      <c r="CS10" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT10" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU10" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV10" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CW10" s="71">
         <f>IFERROR((VLOOKUP(CQ10,Scoring!$A:$B,2,0))+IF(CS10="y",1,0)+IF(CT10="y",1,0)+IF(CU10="y",1,0)+IF(CV10="y",1,0),0)</f>
         <v>0</v>
@@ -4550,12 +5234,8 @@
       <c r="C11" s="15" t="s">
         <v>395</v>
       </c>
-      <c r="D11" s="24">
-        <v>10.0</v>
-      </c>
-      <c r="E11" s="25">
-        <v>7.0</v>
-      </c>
+      <c r="D11" s="24"/>
+      <c r="E11" s="25"/>
       <c r="F11" s="26" t="s">
         <v>128</v>
       </c>
@@ -4570,14 +5250,10 @@
       </c>
       <c r="J11" s="72">
         <f>IFERROR((VLOOKUP(D11,Scoring!$A:$B,2,0))+IF(F11="y",1,0)+IF(G11="y",1,0)+IF(H11="y",1,0)+IF(I11="y",1,0),0)</f>
-        <v>2</v>
-      </c>
-      <c r="K11" s="24">
-        <v>3.0</v>
-      </c>
-      <c r="L11" s="25">
-        <v>10.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K11" s="24"/>
+      <c r="L11" s="25"/>
       <c r="M11" s="26" t="s">
         <v>128</v>
       </c>
@@ -4592,14 +5268,10 @@
       </c>
       <c r="Q11" s="72">
         <f>IFERROR((VLOOKUP(K11,Scoring!$A:$B,2,0))+IF(M11="y",1,0)+IF(N11="y",1,0)+IF(O11="y",1,0)+IF(P11="y",1,0),0)</f>
-        <v>15</v>
-      </c>
-      <c r="R11" s="24">
-        <v>13.0</v>
-      </c>
-      <c r="S11" s="25">
-        <v>3.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R11" s="24"/>
+      <c r="S11" s="25"/>
       <c r="T11" s="26" t="s">
         <v>128</v>
       </c>
@@ -4614,114 +5286,202 @@
       </c>
       <c r="X11" s="72">
         <f>IFERROR((VLOOKUP(R11,Scoring!$A:$B,2,0))+IF(T11="y",1,0)+IF(U11="y",1,0)+IF(V11="y",1,0)+IF(W11="y",1,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y11" s="24"/>
       <c r="Z11" s="25"/>
-      <c r="AA11" s="26"/>
-      <c r="AB11" s="27"/>
-      <c r="AC11" s="28"/>
-      <c r="AD11" s="29"/>
+      <c r="AA11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AE11" s="72">
         <f>IFERROR((VLOOKUP(Y11,Scoring!$A:$B,2,0))+IF(AA11="y",1,0)+IF(AB11="y",1,0)+IF(AC11="y",1,0)+IF(AD11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF11" s="24"/>
       <c r="AG11" s="25"/>
-      <c r="AH11" s="26"/>
-      <c r="AI11" s="27"/>
-      <c r="AJ11" s="28"/>
-      <c r="AK11" s="29"/>
+      <c r="AH11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AL11" s="72">
         <f>IFERROR((VLOOKUP(AF11,Scoring!$A:$B,2,0))+IF(AH11="y",1,0)+IF(AI11="y",1,0)+IF(AJ11="y",1,0)+IF(AK11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM11" s="24"/>
       <c r="AN11" s="25"/>
-      <c r="AO11" s="26"/>
-      <c r="AP11" s="27"/>
-      <c r="AQ11" s="28"/>
-      <c r="AR11" s="29"/>
+      <c r="AO11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AS11" s="72">
         <f>IFERROR((VLOOKUP(AM11,Scoring!$A:$B,2,0))+IF(AO11="y",1,0)+IF(AP11="y",1,0)+IF(AQ11="y",1,0)+IF(AR11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT11" s="24"/>
       <c r="AU11" s="25"/>
-      <c r="AV11" s="26"/>
-      <c r="AW11" s="27"/>
-      <c r="AX11" s="28"/>
-      <c r="AY11" s="29"/>
+      <c r="AV11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ11" s="72">
         <f>IFERROR((VLOOKUP(AT11,Scoring!$A:$B,2,0))+IF(AV11="y",1,0)+IF(AW11="y",1,0)+IF(AX11="y",1,0)+IF(AY11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA11" s="24"/>
       <c r="BB11" s="25"/>
-      <c r="BC11" s="26"/>
-      <c r="BD11" s="27"/>
-      <c r="BE11" s="28"/>
-      <c r="BF11" s="29"/>
+      <c r="BC11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BG11" s="72">
         <f>IFERROR((VLOOKUP(BA11,Scoring!$A:$B,2,0))+IF(BC11="y",1,0)+IF(BD11="y",1,0)+IF(BE11="y",1,0)+IF(BF11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH11" s="24"/>
       <c r="BI11" s="25"/>
-      <c r="BJ11" s="26"/>
-      <c r="BK11" s="27"/>
-      <c r="BL11" s="28"/>
-      <c r="BM11" s="29"/>
+      <c r="BJ11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BN11" s="72">
         <f>IFERROR((VLOOKUP(BH11,Scoring!$A:$B,2,0))+IF(BJ11="y",1,0)+IF(BK11="y",1,0)+IF(BL11="y",1,0)+IF(BM11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO11" s="24"/>
       <c r="BP11" s="25"/>
-      <c r="BQ11" s="26"/>
-      <c r="BR11" s="27"/>
-      <c r="BS11" s="28"/>
-      <c r="BT11" s="29"/>
+      <c r="BQ11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BU11" s="72">
         <f>IFERROR((VLOOKUP(BO11,Scoring!$A:$B,2,0))+IF(BQ11="y",1,0)+IF(BR11="y",1,0)+IF(BS11="y",1,0)+IF(BT11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV11" s="24"/>
       <c r="BW11" s="25"/>
-      <c r="BX11" s="26"/>
-      <c r="BY11" s="27"/>
-      <c r="BZ11" s="28"/>
-      <c r="CA11" s="29"/>
+      <c r="BX11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CB11" s="72">
         <f>IFERROR((VLOOKUP(BV11,Scoring!$A:$B,2,0))+IF(BX11="y",1,0)+IF(BY11="y",1,0)+IF(BZ11="y",1,0)+IF(CA11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC11" s="24"/>
       <c r="CD11" s="25"/>
-      <c r="CE11" s="26"/>
-      <c r="CF11" s="27"/>
-      <c r="CG11" s="28"/>
-      <c r="CH11" s="29"/>
+      <c r="CE11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CI11" s="72">
         <f>IFERROR((VLOOKUP(CC11,Scoring!$A:$B,2,0))+IF(CE11="y",1,0)+IF(CF11="y",1,0)+IF(CG11="y",1,0)+IF(CH11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ11" s="24"/>
       <c r="CK11" s="25"/>
-      <c r="CL11" s="26"/>
-      <c r="CM11" s="27"/>
-      <c r="CN11" s="28"/>
-      <c r="CO11" s="29"/>
+      <c r="CL11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CP11" s="72">
         <f>IFERROR((VLOOKUP(CJ11,Scoring!$A:$B,2,0))+IF(CL11="y",1,0)+IF(CM11="y",1,0)+IF(CN11="y",1,0)+IF(CO11="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ11" s="24"/>
       <c r="CR11" s="25"/>
-      <c r="CS11" s="26"/>
-      <c r="CT11" s="27"/>
-      <c r="CU11" s="28"/>
-      <c r="CV11" s="29"/>
+      <c r="CS11" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT11" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU11" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV11" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CW11" s="72">
         <f>IFERROR((VLOOKUP(CQ11,Scoring!$A:$B,2,0))+IF(CS11="y",1,0)+IF(CT11="y",1,0)+IF(CU11="y",1,0)+IF(CV11="y",1,0),0)</f>
         <v>0</v>
@@ -4740,12 +5500,8 @@
       <c r="C12" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="36">
-        <v>11.0</v>
-      </c>
-      <c r="E12" s="37">
-        <v>6.0</v>
-      </c>
+      <c r="D12" s="36"/>
+      <c r="E12" s="37"/>
       <c r="F12" s="38" t="s">
         <v>128</v>
       </c>
@@ -4760,14 +5516,10 @@
       </c>
       <c r="J12" s="71">
         <f>IFERROR((VLOOKUP(D12,Scoring!$A:$B,2,0))+IF(F12="y",1,0)+IF(G12="y",1,0)+IF(H12="y",1,0)+IF(I12="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="K12" s="36">
-        <v>5.0</v>
-      </c>
-      <c r="L12" s="37">
-        <v>11.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K12" s="36"/>
+      <c r="L12" s="37"/>
       <c r="M12" s="38" t="s">
         <v>128</v>
       </c>
@@ -4782,14 +5534,10 @@
       </c>
       <c r="Q12" s="71">
         <f>IFERROR((VLOOKUP(K12,Scoring!$A:$B,2,0))+IF(M12="y",1,0)+IF(N12="y",1,0)+IF(O12="y",1,0)+IF(P12="y",1,0),0)</f>
-        <v>10</v>
-      </c>
-      <c r="R12" s="36">
-        <v>11.0</v>
-      </c>
-      <c r="S12" s="37">
-        <v>5.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R12" s="36"/>
+      <c r="S12" s="37"/>
       <c r="T12" s="38" t="s">
         <v>128</v>
       </c>
@@ -4804,114 +5552,202 @@
       </c>
       <c r="X12" s="71">
         <f>IFERROR((VLOOKUP(R12,Scoring!$A:$B,2,0))+IF(T12="y",1,0)+IF(U12="y",1,0)+IF(V12="y",1,0)+IF(W12="y",1,0),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="36"/>
       <c r="Z12" s="37"/>
-      <c r="AA12" s="38"/>
-      <c r="AB12" s="39"/>
-      <c r="AC12" s="40"/>
-      <c r="AD12" s="41"/>
+      <c r="AA12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AE12" s="71">
         <f>IFERROR((VLOOKUP(Y12,Scoring!$A:$B,2,0))+IF(AA12="y",1,0)+IF(AB12="y",1,0)+IF(AC12="y",1,0)+IF(AD12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF12" s="36"/>
       <c r="AG12" s="37"/>
-      <c r="AH12" s="38"/>
-      <c r="AI12" s="39"/>
-      <c r="AJ12" s="40"/>
-      <c r="AK12" s="41"/>
+      <c r="AH12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AL12" s="71">
         <f>IFERROR((VLOOKUP(AF12,Scoring!$A:$B,2,0))+IF(AH12="y",1,0)+IF(AI12="y",1,0)+IF(AJ12="y",1,0)+IF(AK12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM12" s="36"/>
       <c r="AN12" s="37"/>
-      <c r="AO12" s="38"/>
-      <c r="AP12" s="39"/>
-      <c r="AQ12" s="40"/>
-      <c r="AR12" s="41"/>
+      <c r="AO12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AS12" s="71">
         <f>IFERROR((VLOOKUP(AM12,Scoring!$A:$B,2,0))+IF(AO12="y",1,0)+IF(AP12="y",1,0)+IF(AQ12="y",1,0)+IF(AR12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT12" s="36"/>
       <c r="AU12" s="37"/>
-      <c r="AV12" s="38"/>
-      <c r="AW12" s="39"/>
-      <c r="AX12" s="40"/>
-      <c r="AY12" s="41"/>
+      <c r="AV12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ12" s="71">
         <f>IFERROR((VLOOKUP(AT12,Scoring!$A:$B,2,0))+IF(AV12="y",1,0)+IF(AW12="y",1,0)+IF(AX12="y",1,0)+IF(AY12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA12" s="36"/>
       <c r="BB12" s="37"/>
-      <c r="BC12" s="38"/>
-      <c r="BD12" s="39"/>
-      <c r="BE12" s="40"/>
-      <c r="BF12" s="41"/>
+      <c r="BC12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BG12" s="71">
         <f>IFERROR((VLOOKUP(BA12,Scoring!$A:$B,2,0))+IF(BC12="y",1,0)+IF(BD12="y",1,0)+IF(BE12="y",1,0)+IF(BF12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH12" s="36"/>
       <c r="BI12" s="37"/>
-      <c r="BJ12" s="38"/>
-      <c r="BK12" s="39"/>
-      <c r="BL12" s="40"/>
-      <c r="BM12" s="41"/>
+      <c r="BJ12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BN12" s="71">
         <f>IFERROR((VLOOKUP(BH12,Scoring!$A:$B,2,0))+IF(BJ12="y",1,0)+IF(BK12="y",1,0)+IF(BL12="y",1,0)+IF(BM12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO12" s="36"/>
       <c r="BP12" s="37"/>
-      <c r="BQ12" s="38"/>
-      <c r="BR12" s="39"/>
-      <c r="BS12" s="40"/>
-      <c r="BT12" s="41"/>
+      <c r="BQ12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BU12" s="71">
         <f>IFERROR((VLOOKUP(BO12,Scoring!$A:$B,2,0))+IF(BQ12="y",1,0)+IF(BR12="y",1,0)+IF(BS12="y",1,0)+IF(BT12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV12" s="36"/>
       <c r="BW12" s="37"/>
-      <c r="BX12" s="38"/>
-      <c r="BY12" s="39"/>
-      <c r="BZ12" s="40"/>
-      <c r="CA12" s="41"/>
+      <c r="BX12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CB12" s="71">
         <f>IFERROR((VLOOKUP(BV12,Scoring!$A:$B,2,0))+IF(BX12="y",1,0)+IF(BY12="y",1,0)+IF(BZ12="y",1,0)+IF(CA12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC12" s="36"/>
       <c r="CD12" s="37"/>
-      <c r="CE12" s="38"/>
-      <c r="CF12" s="39"/>
-      <c r="CG12" s="40"/>
-      <c r="CH12" s="41"/>
+      <c r="CE12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CI12" s="71">
         <f>IFERROR((VLOOKUP(CC12,Scoring!$A:$B,2,0))+IF(CE12="y",1,0)+IF(CF12="y",1,0)+IF(CG12="y",1,0)+IF(CH12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ12" s="36"/>
       <c r="CK12" s="37"/>
-      <c r="CL12" s="38"/>
-      <c r="CM12" s="39"/>
-      <c r="CN12" s="40"/>
-      <c r="CO12" s="41"/>
+      <c r="CL12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CP12" s="71">
         <f>IFERROR((VLOOKUP(CJ12,Scoring!$A:$B,2,0))+IF(CL12="y",1,0)+IF(CM12="y",1,0)+IF(CN12="y",1,0)+IF(CO12="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ12" s="36"/>
       <c r="CR12" s="37"/>
-      <c r="CS12" s="38"/>
-      <c r="CT12" s="39"/>
-      <c r="CU12" s="40"/>
-      <c r="CV12" s="41"/>
+      <c r="CS12" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT12" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV12" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CW12" s="71">
         <f>IFERROR((VLOOKUP(CQ12,Scoring!$A:$B,2,0))+IF(CS12="y",1,0)+IF(CT12="y",1,0)+IF(CU12="y",1,0)+IF(CV12="y",1,0),0)</f>
         <v>0</v>
@@ -4930,12 +5766,8 @@
       <c r="C13" s="15" t="s">
         <v>395</v>
       </c>
-      <c r="D13" s="24">
-        <v>12.0</v>
-      </c>
-      <c r="E13" s="25">
-        <v>5.0</v>
-      </c>
+      <c r="D13" s="24"/>
+      <c r="E13" s="25"/>
       <c r="F13" s="26" t="s">
         <v>128</v>
       </c>
@@ -4950,14 +5782,10 @@
       </c>
       <c r="J13" s="72">
         <f>IFERROR((VLOOKUP(D13,Scoring!$A:$B,2,0))+IF(F13="y",1,0)+IF(G13="y",1,0)+IF(H13="y",1,0)+IF(I13="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="K13" s="24">
-        <v>7.0</v>
-      </c>
-      <c r="L13" s="25">
-        <v>12.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K13" s="24"/>
+      <c r="L13" s="25"/>
       <c r="M13" s="26" t="s">
         <v>128</v>
       </c>
@@ -4972,14 +5800,10 @@
       </c>
       <c r="Q13" s="72">
         <f>IFERROR((VLOOKUP(K13,Scoring!$A:$B,2,0))+IF(M13="y",1,0)+IF(N13="y",1,0)+IF(O13="y",1,0)+IF(P13="y",1,0),0)</f>
-        <v>6</v>
-      </c>
-      <c r="R13" s="24">
-        <v>9.0</v>
-      </c>
-      <c r="S13" s="25">
-        <v>7.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R13" s="24"/>
+      <c r="S13" s="25"/>
       <c r="T13" s="26" t="s">
         <v>128</v>
       </c>
@@ -4994,114 +5818,202 @@
       </c>
       <c r="X13" s="72">
         <f>IFERROR((VLOOKUP(R13,Scoring!$A:$B,2,0))+IF(T13="y",1,0)+IF(U13="y",1,0)+IF(V13="y",1,0)+IF(W13="y",1,0),0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Y13" s="24"/>
       <c r="Z13" s="25"/>
-      <c r="AA13" s="26"/>
-      <c r="AB13" s="27"/>
-      <c r="AC13" s="28"/>
-      <c r="AD13" s="29"/>
+      <c r="AA13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AE13" s="72">
         <f>IFERROR((VLOOKUP(Y13,Scoring!$A:$B,2,0))+IF(AA13="y",1,0)+IF(AB13="y",1,0)+IF(AC13="y",1,0)+IF(AD13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF13" s="24"/>
       <c r="AG13" s="25"/>
-      <c r="AH13" s="26"/>
-      <c r="AI13" s="27"/>
-      <c r="AJ13" s="28"/>
-      <c r="AK13" s="29"/>
+      <c r="AH13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AL13" s="72">
         <f>IFERROR((VLOOKUP(AF13,Scoring!$A:$B,2,0))+IF(AH13="y",1,0)+IF(AI13="y",1,0)+IF(AJ13="y",1,0)+IF(AK13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM13" s="24"/>
       <c r="AN13" s="25"/>
-      <c r="AO13" s="26"/>
-      <c r="AP13" s="27"/>
-      <c r="AQ13" s="28"/>
-      <c r="AR13" s="29"/>
+      <c r="AO13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AS13" s="72">
         <f>IFERROR((VLOOKUP(AM13,Scoring!$A:$B,2,0))+IF(AO13="y",1,0)+IF(AP13="y",1,0)+IF(AQ13="y",1,0)+IF(AR13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT13" s="24"/>
       <c r="AU13" s="25"/>
-      <c r="AV13" s="26"/>
-      <c r="AW13" s="27"/>
-      <c r="AX13" s="28"/>
-      <c r="AY13" s="29"/>
+      <c r="AV13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ13" s="72">
         <f>IFERROR((VLOOKUP(AT13,Scoring!$A:$B,2,0))+IF(AV13="y",1,0)+IF(AW13="y",1,0)+IF(AX13="y",1,0)+IF(AY13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA13" s="24"/>
       <c r="BB13" s="25"/>
-      <c r="BC13" s="26"/>
-      <c r="BD13" s="27"/>
-      <c r="BE13" s="28"/>
-      <c r="BF13" s="29"/>
+      <c r="BC13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BG13" s="72">
         <f>IFERROR((VLOOKUP(BA13,Scoring!$A:$B,2,0))+IF(BC13="y",1,0)+IF(BD13="y",1,0)+IF(BE13="y",1,0)+IF(BF13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH13" s="24"/>
       <c r="BI13" s="25"/>
-      <c r="BJ13" s="26"/>
-      <c r="BK13" s="27"/>
-      <c r="BL13" s="28"/>
-      <c r="BM13" s="29"/>
+      <c r="BJ13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BN13" s="72">
         <f>IFERROR((VLOOKUP(BH13,Scoring!$A:$B,2,0))+IF(BJ13="y",1,0)+IF(BK13="y",1,0)+IF(BL13="y",1,0)+IF(BM13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO13" s="24"/>
       <c r="BP13" s="25"/>
-      <c r="BQ13" s="26"/>
-      <c r="BR13" s="27"/>
-      <c r="BS13" s="28"/>
-      <c r="BT13" s="29"/>
+      <c r="BQ13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BU13" s="72">
         <f>IFERROR((VLOOKUP(BO13,Scoring!$A:$B,2,0))+IF(BQ13="y",1,0)+IF(BR13="y",1,0)+IF(BS13="y",1,0)+IF(BT13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV13" s="24"/>
       <c r="BW13" s="25"/>
-      <c r="BX13" s="26"/>
-      <c r="BY13" s="27"/>
-      <c r="BZ13" s="28"/>
-      <c r="CA13" s="29"/>
+      <c r="BX13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CB13" s="72">
         <f>IFERROR((VLOOKUP(BV13,Scoring!$A:$B,2,0))+IF(BX13="y",1,0)+IF(BY13="y",1,0)+IF(BZ13="y",1,0)+IF(CA13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC13" s="24"/>
       <c r="CD13" s="25"/>
-      <c r="CE13" s="26"/>
-      <c r="CF13" s="27"/>
-      <c r="CG13" s="28"/>
-      <c r="CH13" s="29"/>
+      <c r="CE13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CI13" s="72">
         <f>IFERROR((VLOOKUP(CC13,Scoring!$A:$B,2,0))+IF(CE13="y",1,0)+IF(CF13="y",1,0)+IF(CG13="y",1,0)+IF(CH13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ13" s="24"/>
       <c r="CK13" s="25"/>
-      <c r="CL13" s="26"/>
-      <c r="CM13" s="27"/>
-      <c r="CN13" s="28"/>
-      <c r="CO13" s="29"/>
+      <c r="CL13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CP13" s="72">
         <f>IFERROR((VLOOKUP(CJ13,Scoring!$A:$B,2,0))+IF(CL13="y",1,0)+IF(CM13="y",1,0)+IF(CN13="y",1,0)+IF(CO13="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ13" s="24"/>
       <c r="CR13" s="25"/>
-      <c r="CS13" s="26"/>
-      <c r="CT13" s="27"/>
-      <c r="CU13" s="28"/>
-      <c r="CV13" s="29"/>
+      <c r="CS13" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT13" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU13" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV13" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CW13" s="72">
         <f>IFERROR((VLOOKUP(CQ13,Scoring!$A:$B,2,0))+IF(CS13="y",1,0)+IF(CT13="y",1,0)+IF(CU13="y",1,0)+IF(CV13="y",1,0),0)</f>
         <v>0</v>
@@ -5120,12 +6032,8 @@
       <c r="C14" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="36">
-        <v>13.0</v>
-      </c>
-      <c r="E14" s="37">
-        <v>4.0</v>
-      </c>
+      <c r="D14" s="36"/>
+      <c r="E14" s="37"/>
       <c r="F14" s="38" t="s">
         <v>128</v>
       </c>
@@ -5140,14 +6048,10 @@
       </c>
       <c r="J14" s="71">
         <f>IFERROR((VLOOKUP(D14,Scoring!$A:$B,2,0))+IF(F14="y",1,0)+IF(G14="y",1,0)+IF(H14="y",1,0)+IF(I14="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="K14" s="36">
-        <v>9.0</v>
-      </c>
-      <c r="L14" s="37">
-        <v>13.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K14" s="36"/>
+      <c r="L14" s="37"/>
       <c r="M14" s="38" t="s">
         <v>128</v>
       </c>
@@ -5162,14 +6066,10 @@
       </c>
       <c r="Q14" s="71">
         <f>IFERROR((VLOOKUP(K14,Scoring!$A:$B,2,0))+IF(M14="y",1,0)+IF(N14="y",1,0)+IF(O14="y",1,0)+IF(P14="y",1,0),0)</f>
-        <v>3</v>
-      </c>
-      <c r="R14" s="36">
-        <v>7.0</v>
-      </c>
-      <c r="S14" s="37">
-        <v>9.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R14" s="36"/>
+      <c r="S14" s="37"/>
       <c r="T14" s="38" t="s">
         <v>128</v>
       </c>
@@ -5184,114 +6084,202 @@
       </c>
       <c r="X14" s="71">
         <f>IFERROR((VLOOKUP(R14,Scoring!$A:$B,2,0))+IF(T14="y",1,0)+IF(U14="y",1,0)+IF(V14="y",1,0)+IF(W14="y",1,0),0)</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Y14" s="36"/>
       <c r="Z14" s="37"/>
-      <c r="AA14" s="38"/>
-      <c r="AB14" s="39"/>
-      <c r="AC14" s="40"/>
-      <c r="AD14" s="41"/>
+      <c r="AA14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AE14" s="71">
         <f>IFERROR((VLOOKUP(Y14,Scoring!$A:$B,2,0))+IF(AA14="y",1,0)+IF(AB14="y",1,0)+IF(AC14="y",1,0)+IF(AD14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF14" s="36"/>
       <c r="AG14" s="37"/>
-      <c r="AH14" s="38"/>
-      <c r="AI14" s="39"/>
-      <c r="AJ14" s="40"/>
-      <c r="AK14" s="41"/>
+      <c r="AH14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AL14" s="71">
         <f>IFERROR((VLOOKUP(AF14,Scoring!$A:$B,2,0))+IF(AH14="y",1,0)+IF(AI14="y",1,0)+IF(AJ14="y",1,0)+IF(AK14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM14" s="36"/>
       <c r="AN14" s="37"/>
-      <c r="AO14" s="38"/>
-      <c r="AP14" s="39"/>
-      <c r="AQ14" s="40"/>
-      <c r="AR14" s="41"/>
+      <c r="AO14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AS14" s="71">
         <f>IFERROR((VLOOKUP(AM14,Scoring!$A:$B,2,0))+IF(AO14="y",1,0)+IF(AP14="y",1,0)+IF(AQ14="y",1,0)+IF(AR14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT14" s="36"/>
       <c r="AU14" s="37"/>
-      <c r="AV14" s="38"/>
-      <c r="AW14" s="39"/>
-      <c r="AX14" s="40"/>
-      <c r="AY14" s="41"/>
+      <c r="AV14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ14" s="71">
         <f>IFERROR((VLOOKUP(AT14,Scoring!$A:$B,2,0))+IF(AV14="y",1,0)+IF(AW14="y",1,0)+IF(AX14="y",1,0)+IF(AY14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA14" s="36"/>
       <c r="BB14" s="37"/>
-      <c r="BC14" s="38"/>
-      <c r="BD14" s="39"/>
-      <c r="BE14" s="40"/>
-      <c r="BF14" s="41"/>
+      <c r="BC14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BG14" s="71">
         <f>IFERROR((VLOOKUP(BA14,Scoring!$A:$B,2,0))+IF(BC14="y",1,0)+IF(BD14="y",1,0)+IF(BE14="y",1,0)+IF(BF14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH14" s="36"/>
       <c r="BI14" s="37"/>
-      <c r="BJ14" s="38"/>
-      <c r="BK14" s="39"/>
-      <c r="BL14" s="40"/>
-      <c r="BM14" s="41"/>
+      <c r="BJ14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BN14" s="71">
         <f>IFERROR((VLOOKUP(BH14,Scoring!$A:$B,2,0))+IF(BJ14="y",1,0)+IF(BK14="y",1,0)+IF(BL14="y",1,0)+IF(BM14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO14" s="36"/>
       <c r="BP14" s="37"/>
-      <c r="BQ14" s="38"/>
-      <c r="BR14" s="39"/>
-      <c r="BS14" s="40"/>
-      <c r="BT14" s="41"/>
+      <c r="BQ14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="BU14" s="71">
         <f>IFERROR((VLOOKUP(BO14,Scoring!$A:$B,2,0))+IF(BQ14="y",1,0)+IF(BR14="y",1,0)+IF(BS14="y",1,0)+IF(BT14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV14" s="36"/>
       <c r="BW14" s="37"/>
-      <c r="BX14" s="38"/>
-      <c r="BY14" s="39"/>
-      <c r="BZ14" s="40"/>
-      <c r="CA14" s="41"/>
+      <c r="BX14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CB14" s="71">
         <f>IFERROR((VLOOKUP(BV14,Scoring!$A:$B,2,0))+IF(BX14="y",1,0)+IF(BY14="y",1,0)+IF(BZ14="y",1,0)+IF(CA14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC14" s="36"/>
       <c r="CD14" s="37"/>
-      <c r="CE14" s="38"/>
-      <c r="CF14" s="39"/>
-      <c r="CG14" s="40"/>
-      <c r="CH14" s="41"/>
+      <c r="CE14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CI14" s="71">
         <f>IFERROR((VLOOKUP(CC14,Scoring!$A:$B,2,0))+IF(CE14="y",1,0)+IF(CF14="y",1,0)+IF(CG14="y",1,0)+IF(CH14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ14" s="36"/>
       <c r="CK14" s="37"/>
-      <c r="CL14" s="38"/>
-      <c r="CM14" s="39"/>
-      <c r="CN14" s="40"/>
-      <c r="CO14" s="41"/>
+      <c r="CL14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CP14" s="71">
         <f>IFERROR((VLOOKUP(CJ14,Scoring!$A:$B,2,0))+IF(CL14="y",1,0)+IF(CM14="y",1,0)+IF(CN14="y",1,0)+IF(CO14="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ14" s="36"/>
       <c r="CR14" s="37"/>
-      <c r="CS14" s="38"/>
-      <c r="CT14" s="39"/>
-      <c r="CU14" s="40"/>
-      <c r="CV14" s="41"/>
+      <c r="CS14" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT14" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU14" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV14" s="41" t="s">
+        <v>128</v>
+      </c>
       <c r="CW14" s="71">
         <f>IFERROR((VLOOKUP(CQ14,Scoring!$A:$B,2,0))+IF(CS14="y",1,0)+IF(CT14="y",1,0)+IF(CU14="y",1,0)+IF(CV14="y",1,0),0)</f>
         <v>0</v>
@@ -5310,12 +6298,8 @@
       <c r="C15" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="48">
-        <v>23.0</v>
-      </c>
-      <c r="E15" s="49">
-        <v>3.0</v>
-      </c>
+      <c r="D15" s="48"/>
+      <c r="E15" s="49"/>
       <c r="F15" s="50" t="s">
         <v>128</v>
       </c>
@@ -5332,12 +6316,8 @@
         <f>IFERROR((VLOOKUP(D15,Scoring!$A:$B,2,0))+IF(F15="y",1,0)+IF(G15="y",1,0)+IF(H15="y",1,0)+IF(I15="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="48">
-        <v>11.0</v>
-      </c>
-      <c r="L15" s="49">
-        <v>14.0</v>
-      </c>
+      <c r="K15" s="48"/>
+      <c r="L15" s="49"/>
       <c r="M15" s="50" t="s">
         <v>128</v>
       </c>
@@ -5352,14 +6332,10 @@
       </c>
       <c r="Q15" s="72">
         <f>IFERROR((VLOOKUP(K15,Scoring!$A:$B,2,0))+IF(M15="y",1,0)+IF(N15="y",1,0)+IF(O15="y",1,0)+IF(P15="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="R15" s="48">
-        <v>5.0</v>
-      </c>
-      <c r="S15" s="49">
-        <v>11.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R15" s="48"/>
+      <c r="S15" s="49"/>
       <c r="T15" s="50" t="s">
         <v>128</v>
       </c>
@@ -5374,114 +6350,202 @@
       </c>
       <c r="X15" s="72">
         <f>IFERROR((VLOOKUP(R15,Scoring!$A:$B,2,0))+IF(T15="y",1,0)+IF(U15="y",1,0)+IF(V15="y",1,0)+IF(W15="y",1,0),0)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Y15" s="48"/>
       <c r="Z15" s="49"/>
-      <c r="AA15" s="50"/>
-      <c r="AB15" s="51"/>
-      <c r="AC15" s="52"/>
-      <c r="AD15" s="53"/>
+      <c r="AA15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AE15" s="72">
         <f>IFERROR((VLOOKUP(Y15,Scoring!$A:$B,2,0))+IF(AA15="y",1,0)+IF(AB15="y",1,0)+IF(AC15="y",1,0)+IF(AD15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF15" s="48"/>
       <c r="AG15" s="49"/>
-      <c r="AH15" s="50"/>
-      <c r="AI15" s="51"/>
-      <c r="AJ15" s="52"/>
-      <c r="AK15" s="53"/>
+      <c r="AH15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AL15" s="72">
         <f>IFERROR((VLOOKUP(AF15,Scoring!$A:$B,2,0))+IF(AH15="y",1,0)+IF(AI15="y",1,0)+IF(AJ15="y",1,0)+IF(AK15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM15" s="48"/>
       <c r="AN15" s="49"/>
-      <c r="AO15" s="50"/>
-      <c r="AP15" s="51"/>
-      <c r="AQ15" s="52"/>
-      <c r="AR15" s="53"/>
+      <c r="AO15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AS15" s="72">
         <f>IFERROR((VLOOKUP(AM15,Scoring!$A:$B,2,0))+IF(AO15="y",1,0)+IF(AP15="y",1,0)+IF(AQ15="y",1,0)+IF(AR15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT15" s="48"/>
       <c r="AU15" s="49"/>
-      <c r="AV15" s="50"/>
-      <c r="AW15" s="51"/>
-      <c r="AX15" s="52"/>
-      <c r="AY15" s="53"/>
+      <c r="AV15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ15" s="72">
         <f>IFERROR((VLOOKUP(AT15,Scoring!$A:$B,2,0))+IF(AV15="y",1,0)+IF(AW15="y",1,0)+IF(AX15="y",1,0)+IF(AY15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA15" s="48"/>
       <c r="BB15" s="49"/>
-      <c r="BC15" s="50"/>
-      <c r="BD15" s="51"/>
-      <c r="BE15" s="52"/>
-      <c r="BF15" s="53"/>
+      <c r="BC15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BG15" s="72">
         <f>IFERROR((VLOOKUP(BA15,Scoring!$A:$B,2,0))+IF(BC15="y",1,0)+IF(BD15="y",1,0)+IF(BE15="y",1,0)+IF(BF15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH15" s="48"/>
       <c r="BI15" s="49"/>
-      <c r="BJ15" s="50"/>
-      <c r="BK15" s="51"/>
-      <c r="BL15" s="52"/>
-      <c r="BM15" s="53"/>
+      <c r="BJ15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BN15" s="72">
         <f>IFERROR((VLOOKUP(BH15,Scoring!$A:$B,2,0))+IF(BJ15="y",1,0)+IF(BK15="y",1,0)+IF(BL15="y",1,0)+IF(BM15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO15" s="48"/>
       <c r="BP15" s="49"/>
-      <c r="BQ15" s="50"/>
-      <c r="BR15" s="51"/>
-      <c r="BS15" s="52"/>
-      <c r="BT15" s="53"/>
+      <c r="BQ15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="BU15" s="72">
         <f>IFERROR((VLOOKUP(BO15,Scoring!$A:$B,2,0))+IF(BQ15="y",1,0)+IF(BR15="y",1,0)+IF(BS15="y",1,0)+IF(BT15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV15" s="48"/>
       <c r="BW15" s="49"/>
-      <c r="BX15" s="50"/>
-      <c r="BY15" s="51"/>
-      <c r="BZ15" s="52"/>
-      <c r="CA15" s="53"/>
+      <c r="BX15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CB15" s="72">
         <f>IFERROR((VLOOKUP(BV15,Scoring!$A:$B,2,0))+IF(BX15="y",1,0)+IF(BY15="y",1,0)+IF(BZ15="y",1,0)+IF(CA15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC15" s="48"/>
       <c r="CD15" s="49"/>
-      <c r="CE15" s="50"/>
-      <c r="CF15" s="51"/>
-      <c r="CG15" s="52"/>
-      <c r="CH15" s="53"/>
+      <c r="CE15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CI15" s="72">
         <f>IFERROR((VLOOKUP(CC15,Scoring!$A:$B,2,0))+IF(CE15="y",1,0)+IF(CF15="y",1,0)+IF(CG15="y",1,0)+IF(CH15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ15" s="48"/>
       <c r="CK15" s="49"/>
-      <c r="CL15" s="50"/>
-      <c r="CM15" s="51"/>
-      <c r="CN15" s="52"/>
-      <c r="CO15" s="53"/>
+      <c r="CL15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CP15" s="72">
         <f>IFERROR((VLOOKUP(CJ15,Scoring!$A:$B,2,0))+IF(CL15="y",1,0)+IF(CM15="y",1,0)+IF(CN15="y",1,0)+IF(CO15="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ15" s="48"/>
       <c r="CR15" s="49"/>
-      <c r="CS15" s="50"/>
-      <c r="CT15" s="51"/>
-      <c r="CU15" s="52"/>
-      <c r="CV15" s="53"/>
+      <c r="CS15" s="50" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT15" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV15" s="53" t="s">
+        <v>128</v>
+      </c>
       <c r="CW15" s="72">
         <f>IFERROR((VLOOKUP(CQ15,Scoring!$A:$B,2,0))+IF(CS15="y",1,0)+IF(CT15="y",1,0)+IF(CU15="y",1,0)+IF(CV15="y",1,0),0)</f>
         <v>0</v>
@@ -5500,12 +6564,8 @@
       <c r="C16" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="24">
-        <v>24.0</v>
-      </c>
-      <c r="E16" s="25">
-        <v>2.0</v>
-      </c>
+      <c r="D16" s="24"/>
+      <c r="E16" s="25"/>
       <c r="F16" s="26" t="s">
         <v>128</v>
       </c>
@@ -5522,12 +6582,8 @@
         <f>IFERROR((VLOOKUP(D16,Scoring!$A:$B,2,0))+IF(F16="y",1,0)+IF(G16="y",1,0)+IF(H16="y",1,0)+IF(I16="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="K16" s="24">
-        <v>13.0</v>
-      </c>
-      <c r="L16" s="25">
-        <v>15.0</v>
-      </c>
+      <c r="K16" s="24"/>
+      <c r="L16" s="25"/>
       <c r="M16" s="26" t="s">
         <v>128</v>
       </c>
@@ -5542,14 +6598,10 @@
       </c>
       <c r="Q16" s="71">
         <f>IFERROR((VLOOKUP(K16,Scoring!$A:$B,2,0))+IF(M16="y",1,0)+IF(N16="y",1,0)+IF(O16="y",1,0)+IF(P16="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="R16" s="24">
-        <v>3.0</v>
-      </c>
-      <c r="S16" s="25">
-        <v>13.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R16" s="24"/>
+      <c r="S16" s="25"/>
       <c r="T16" s="26" t="s">
         <v>128</v>
       </c>
@@ -5564,114 +6616,202 @@
       </c>
       <c r="X16" s="71">
         <f>IFERROR((VLOOKUP(R16,Scoring!$A:$B,2,0))+IF(T16="y",1,0)+IF(U16="y",1,0)+IF(V16="y",1,0)+IF(W16="y",1,0),0)</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="Y16" s="24"/>
       <c r="Z16" s="25"/>
-      <c r="AA16" s="26"/>
-      <c r="AB16" s="27"/>
-      <c r="AC16" s="28"/>
-      <c r="AD16" s="29"/>
+      <c r="AA16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AE16" s="71">
         <f>IFERROR((VLOOKUP(Y16,Scoring!$A:$B,2,0))+IF(AA16="y",1,0)+IF(AB16="y",1,0)+IF(AC16="y",1,0)+IF(AD16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF16" s="24"/>
       <c r="AG16" s="25"/>
-      <c r="AH16" s="26"/>
-      <c r="AI16" s="27"/>
-      <c r="AJ16" s="28"/>
-      <c r="AK16" s="29"/>
+      <c r="AH16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AL16" s="71">
         <f>IFERROR((VLOOKUP(AF16,Scoring!$A:$B,2,0))+IF(AH16="y",1,0)+IF(AI16="y",1,0)+IF(AJ16="y",1,0)+IF(AK16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM16" s="24"/>
       <c r="AN16" s="25"/>
-      <c r="AO16" s="26"/>
-      <c r="AP16" s="27"/>
-      <c r="AQ16" s="28"/>
-      <c r="AR16" s="29"/>
+      <c r="AO16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AS16" s="71">
         <f>IFERROR((VLOOKUP(AM16,Scoring!$A:$B,2,0))+IF(AO16="y",1,0)+IF(AP16="y",1,0)+IF(AQ16="y",1,0)+IF(AR16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT16" s="24"/>
       <c r="AU16" s="25"/>
-      <c r="AV16" s="26"/>
-      <c r="AW16" s="27"/>
-      <c r="AX16" s="28"/>
-      <c r="AY16" s="29"/>
+      <c r="AV16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ16" s="71">
         <f>IFERROR((VLOOKUP(AT16,Scoring!$A:$B,2,0))+IF(AV16="y",1,0)+IF(AW16="y",1,0)+IF(AX16="y",1,0)+IF(AY16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA16" s="24"/>
       <c r="BB16" s="25"/>
-      <c r="BC16" s="26"/>
-      <c r="BD16" s="27"/>
-      <c r="BE16" s="28"/>
-      <c r="BF16" s="29"/>
+      <c r="BC16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BG16" s="71">
         <f>IFERROR((VLOOKUP(BA16,Scoring!$A:$B,2,0))+IF(BC16="y",1,0)+IF(BD16="y",1,0)+IF(BE16="y",1,0)+IF(BF16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH16" s="24"/>
       <c r="BI16" s="25"/>
-      <c r="BJ16" s="26"/>
-      <c r="BK16" s="27"/>
-      <c r="BL16" s="28"/>
-      <c r="BM16" s="29"/>
+      <c r="BJ16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BN16" s="71">
         <f>IFERROR((VLOOKUP(BH16,Scoring!$A:$B,2,0))+IF(BJ16="y",1,0)+IF(BK16="y",1,0)+IF(BL16="y",1,0)+IF(BM16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO16" s="24"/>
       <c r="BP16" s="25"/>
-      <c r="BQ16" s="26"/>
-      <c r="BR16" s="27"/>
-      <c r="BS16" s="28"/>
-      <c r="BT16" s="29"/>
+      <c r="BQ16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="BU16" s="71">
         <f>IFERROR((VLOOKUP(BO16,Scoring!$A:$B,2,0))+IF(BQ16="y",1,0)+IF(BR16="y",1,0)+IF(BS16="y",1,0)+IF(BT16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV16" s="24"/>
       <c r="BW16" s="25"/>
-      <c r="BX16" s="26"/>
-      <c r="BY16" s="27"/>
-      <c r="BZ16" s="28"/>
-      <c r="CA16" s="29"/>
+      <c r="BX16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CB16" s="71">
         <f>IFERROR((VLOOKUP(BV16,Scoring!$A:$B,2,0))+IF(BX16="y",1,0)+IF(BY16="y",1,0)+IF(BZ16="y",1,0)+IF(CA16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC16" s="24"/>
       <c r="CD16" s="25"/>
-      <c r="CE16" s="26"/>
-      <c r="CF16" s="27"/>
-      <c r="CG16" s="28"/>
-      <c r="CH16" s="29"/>
+      <c r="CE16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CI16" s="71">
         <f>IFERROR((VLOOKUP(CC16,Scoring!$A:$B,2,0))+IF(CE16="y",1,0)+IF(CF16="y",1,0)+IF(CG16="y",1,0)+IF(CH16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ16" s="24"/>
       <c r="CK16" s="25"/>
-      <c r="CL16" s="26"/>
-      <c r="CM16" s="27"/>
-      <c r="CN16" s="28"/>
-      <c r="CO16" s="29"/>
+      <c r="CL16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CP16" s="71">
         <f>IFERROR((VLOOKUP(CJ16,Scoring!$A:$B,2,0))+IF(CL16="y",1,0)+IF(CM16="y",1,0)+IF(CN16="y",1,0)+IF(CO16="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ16" s="24"/>
       <c r="CR16" s="25"/>
-      <c r="CS16" s="26"/>
-      <c r="CT16" s="27"/>
-      <c r="CU16" s="28"/>
-      <c r="CV16" s="29"/>
+      <c r="CS16" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT16" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU16" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV16" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="CW16" s="71">
         <f>IFERROR((VLOOKUP(CQ16,Scoring!$A:$B,2,0))+IF(CS16="y",1,0)+IF(CT16="y",1,0)+IF(CU16="y",1,0)+IF(CV16="y",1,0),0)</f>
         <v>0</v>
@@ -5690,12 +6830,8 @@
       <c r="C17" s="59" t="s">
         <v>395</v>
       </c>
-      <c r="D17" s="60">
-        <v>25.0</v>
-      </c>
-      <c r="E17" s="61">
-        <v>1.0</v>
-      </c>
+      <c r="D17" s="60"/>
+      <c r="E17" s="61"/>
       <c r="F17" s="62" t="s">
         <v>128</v>
       </c>
@@ -5712,12 +6848,8 @@
         <f>IFERROR((VLOOKUP(D17,Scoring!$A:$B,2,0))+IF(F17="y",1,0)+IF(G17="y",1,0)+IF(H17="y",1,0)+IF(I17="y",1,0),0)</f>
         <v>0</v>
       </c>
-      <c r="K17" s="60">
-        <v>15.0</v>
-      </c>
-      <c r="L17" s="61">
-        <v>16.0</v>
-      </c>
+      <c r="K17" s="60"/>
+      <c r="L17" s="61"/>
       <c r="M17" s="62" t="s">
         <v>128</v>
       </c>
@@ -5732,14 +6864,10 @@
       </c>
       <c r="Q17" s="73">
         <f>IFERROR((VLOOKUP(K17,Scoring!$A:$B,2,0))+IF(M17="y",1,0)+IF(N17="y",1,0)+IF(O17="y",1,0)+IF(P17="y",1,0),0)</f>
-        <v>1</v>
-      </c>
-      <c r="R17" s="60">
-        <v>1.0</v>
-      </c>
-      <c r="S17" s="61">
-        <v>15.0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="R17" s="60"/>
+      <c r="S17" s="61"/>
       <c r="T17" s="62" t="s">
         <v>128</v>
       </c>
@@ -5754,114 +6882,202 @@
       </c>
       <c r="X17" s="73">
         <f>IFERROR((VLOOKUP(R17,Scoring!$A:$B,2,0))+IF(T17="y",1,0)+IF(U17="y",1,0)+IF(V17="y",1,0)+IF(W17="y",1,0),0)</f>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="Y17" s="60"/>
       <c r="Z17" s="61"/>
-      <c r="AA17" s="62"/>
-      <c r="AB17" s="63"/>
-      <c r="AC17" s="64"/>
-      <c r="AD17" s="65"/>
+      <c r="AA17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="AB17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="AD17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="AE17" s="73">
         <f>IFERROR((VLOOKUP(Y17,Scoring!$A:$B,2,0))+IF(AA17="y",1,0)+IF(AB17="y",1,0)+IF(AC17="y",1,0)+IF(AD17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AF17" s="60"/>
       <c r="AG17" s="61"/>
-      <c r="AH17" s="62"/>
-      <c r="AI17" s="63"/>
-      <c r="AJ17" s="64"/>
-      <c r="AK17" s="65"/>
+      <c r="AH17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="AJ17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="AK17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="AL17" s="73">
         <f>IFERROR((VLOOKUP(AF17,Scoring!$A:$B,2,0))+IF(AH17="y",1,0)+IF(AI17="y",1,0)+IF(AJ17="y",1,0)+IF(AK17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AM17" s="60"/>
       <c r="AN17" s="61"/>
-      <c r="AO17" s="62"/>
-      <c r="AP17" s="63"/>
-      <c r="AQ17" s="64"/>
-      <c r="AR17" s="65"/>
+      <c r="AO17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="AP17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="AQ17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="AS17" s="73">
         <f>IFERROR((VLOOKUP(AM17,Scoring!$A:$B,2,0))+IF(AO17="y",1,0)+IF(AP17="y",1,0)+IF(AQ17="y",1,0)+IF(AR17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="AT17" s="60"/>
       <c r="AU17" s="61"/>
-      <c r="AV17" s="62"/>
-      <c r="AW17" s="63"/>
-      <c r="AX17" s="64"/>
-      <c r="AY17" s="65"/>
+      <c r="AV17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="AW17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="AX17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="AY17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="AZ17" s="73">
         <f>IFERROR((VLOOKUP(AT17,Scoring!$A:$B,2,0))+IF(AV17="y",1,0)+IF(AW17="y",1,0)+IF(AX17="y",1,0)+IF(AY17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BA17" s="60"/>
       <c r="BB17" s="61"/>
-      <c r="BC17" s="62"/>
-      <c r="BD17" s="63"/>
-      <c r="BE17" s="64"/>
-      <c r="BF17" s="65"/>
+      <c r="BC17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="BD17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="BE17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="BF17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="BG17" s="73">
         <f>IFERROR((VLOOKUP(BA17,Scoring!$A:$B,2,0))+IF(BC17="y",1,0)+IF(BD17="y",1,0)+IF(BE17="y",1,0)+IF(BF17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BH17" s="60"/>
       <c r="BI17" s="61"/>
-      <c r="BJ17" s="62"/>
-      <c r="BK17" s="63"/>
-      <c r="BL17" s="64"/>
-      <c r="BM17" s="65"/>
+      <c r="BJ17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="BK17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="BL17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="BM17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="BN17" s="73">
         <f>IFERROR((VLOOKUP(BH17,Scoring!$A:$B,2,0))+IF(BJ17="y",1,0)+IF(BK17="y",1,0)+IF(BL17="y",1,0)+IF(BM17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BO17" s="60"/>
       <c r="BP17" s="61"/>
-      <c r="BQ17" s="62"/>
-      <c r="BR17" s="63"/>
-      <c r="BS17" s="64"/>
-      <c r="BT17" s="65"/>
+      <c r="BQ17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="BR17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="BS17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="BT17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="BU17" s="73">
         <f>IFERROR((VLOOKUP(BO17,Scoring!$A:$B,2,0))+IF(BQ17="y",1,0)+IF(BR17="y",1,0)+IF(BS17="y",1,0)+IF(BT17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="BV17" s="60"/>
       <c r="BW17" s="61"/>
-      <c r="BX17" s="62"/>
-      <c r="BY17" s="63"/>
-      <c r="BZ17" s="64"/>
-      <c r="CA17" s="65"/>
+      <c r="BX17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="BY17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="BZ17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="CA17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="CB17" s="73">
         <f>IFERROR((VLOOKUP(BV17,Scoring!$A:$B,2,0))+IF(BX17="y",1,0)+IF(BY17="y",1,0)+IF(BZ17="y",1,0)+IF(CA17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CC17" s="60"/>
       <c r="CD17" s="61"/>
-      <c r="CE17" s="62"/>
-      <c r="CF17" s="63"/>
-      <c r="CG17" s="64"/>
-      <c r="CH17" s="65"/>
+      <c r="CE17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="CF17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="CG17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="CH17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="CI17" s="73">
         <f>IFERROR((VLOOKUP(CC17,Scoring!$A:$B,2,0))+IF(CE17="y",1,0)+IF(CF17="y",1,0)+IF(CG17="y",1,0)+IF(CH17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CJ17" s="60"/>
       <c r="CK17" s="61"/>
-      <c r="CL17" s="62"/>
-      <c r="CM17" s="63"/>
-      <c r="CN17" s="64"/>
-      <c r="CO17" s="65"/>
+      <c r="CL17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="CM17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="CN17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="CO17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="CP17" s="73">
         <f>IFERROR((VLOOKUP(CJ17,Scoring!$A:$B,2,0))+IF(CL17="y",1,0)+IF(CM17="y",1,0)+IF(CN17="y",1,0)+IF(CO17="y",1,0),0)</f>
         <v>0</v>
       </c>
       <c r="CQ17" s="60"/>
       <c r="CR17" s="61"/>
-      <c r="CS17" s="62"/>
-      <c r="CT17" s="63"/>
-      <c r="CU17" s="64"/>
-      <c r="CV17" s="65"/>
+      <c r="CS17" s="62" t="s">
+        <v>128</v>
+      </c>
+      <c r="CT17" s="63" t="s">
+        <v>128</v>
+      </c>
+      <c r="CU17" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="CV17" s="65" t="s">
+        <v>128</v>
+      </c>
       <c r="CW17" s="73">
         <f>IFERROR((VLOOKUP(CQ17,Scoring!$A:$B,2,0))+IF(CS17="y",1,0)+IF(CT17="y",1,0)+IF(CU17="y",1,0)+IF(CV17="y",1,0),0)</f>
         <v>0</v>

</xml_diff>

<commit_message>
williams, all time streaks
</commit_message>
<xml_diff>
--- a/the_alternative_f1/The_Alternative_F1.xlsx
+++ b/the_alternative_f1/The_Alternative_F1.xlsx
@@ -9072,7 +9072,7 @@
         <v>0.0</v>
       </c>
       <c r="H3" s="1">
-        <v>0.0</v>
+        <v>22.0</v>
       </c>
       <c r="I3" s="1">
         <v>22.0</v>
@@ -10282,7 +10282,7 @@
         <v>2.0</v>
       </c>
       <c r="H8" s="1">
-        <v>0.0</v>
+        <v>22.0</v>
       </c>
       <c r="I8" s="1">
         <v>22.0</v>
@@ -10524,7 +10524,7 @@
         <v>1.0</v>
       </c>
       <c r="H9" s="1">
-        <v>0.0</v>
+        <v>22.0</v>
       </c>
       <c r="I9" s="1">
         <v>22.0</v>
@@ -10766,7 +10766,7 @@
         <v>0.0</v>
       </c>
       <c r="H10" s="1">
-        <v>0.0</v>
+        <v>22.0</v>
       </c>
       <c r="I10" s="1">
         <v>22.0</v>

</xml_diff>

<commit_message>
updates to latency and power rankings
</commit_message>
<xml_diff>
--- a/the_alternative_f1/The_Alternative_F1.xlsx
+++ b/the_alternative_f1/The_Alternative_F1.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3314" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3320" uniqueCount="428">
   <si>
     <t>Positions</t>
   </si>
@@ -1230,12 +1230,18 @@
     <t>Randy</t>
   </si>
   <si>
-    <t>Pre-Season: TBD</t>
+    <t>Pre-Season: Mexico</t>
   </si>
   <si>
     <t>8/12/2026</t>
   </si>
   <si>
+    <t>Confirmed</t>
+  </si>
+  <si>
+    <t>Pre-Season: Vegas</t>
+  </si>
+  <si>
     <t>8/19/2026</t>
   </si>
   <si>
@@ -1245,67 +1251,40 @@
     <t>8/26/2026</t>
   </si>
   <si>
-    <t>W1</t>
-  </si>
-  <si>
     <t>9/9/2026</t>
   </si>
   <si>
-    <t>W2</t>
+    <t>Imola</t>
   </si>
   <si>
     <t>9/16/2026</t>
   </si>
   <si>
-    <t>W3</t>
-  </si>
-  <si>
     <t>9/30/2026</t>
   </si>
   <si>
-    <t>W4</t>
-  </si>
-  <si>
     <t>10/7/2026</t>
   </si>
   <si>
-    <t>W5</t>
-  </si>
-  <si>
     <t>10/14/2026</t>
   </si>
   <si>
-    <t>W6</t>
-  </si>
-  <si>
     <t>10/28/2026</t>
   </si>
   <si>
-    <t>W7</t>
+    <t>Silverstone Sprint</t>
   </si>
   <si>
     <t>11/4/2026</t>
   </si>
   <si>
-    <t>W8</t>
-  </si>
-  <si>
     <t>11/18/2026</t>
   </si>
   <si>
-    <t>W9</t>
-  </si>
-  <si>
     <t>12/2/2026</t>
   </si>
   <si>
-    <t>W-10</t>
-  </si>
-  <si>
     <t>12/9/2026</t>
-  </si>
-  <si>
-    <t>W-11</t>
   </si>
   <si>
     <t>12/30/2026</t>
@@ -3122,8 +3101,12 @@
       <c r="C2" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="16"/>
-      <c r="E2" s="17"/>
+      <c r="D2" s="16">
+        <v>2.0</v>
+      </c>
+      <c r="E2" s="17">
+        <v>1.0</v>
+      </c>
       <c r="F2" s="18" t="s">
         <v>128</v>
       </c>
@@ -3138,10 +3121,14 @@
       </c>
       <c r="J2" s="85">
         <f>IFERROR((VLOOKUP(D2,Scoring!$A:$B,2,0))+IF(F2="y",1,0)+IF(G2="y",1,0)+IF(H2="y",1,0)+IF(I2="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K2" s="16"/>
-      <c r="L2" s="17"/>
+        <v>18</v>
+      </c>
+      <c r="K2" s="16">
+        <v>3.0</v>
+      </c>
+      <c r="L2" s="17">
+        <v>3.0</v>
+      </c>
       <c r="M2" s="18" t="s">
         <v>128</v>
       </c>
@@ -3156,7 +3143,7 @@
       </c>
       <c r="Q2" s="85">
         <f>IFERROR((VLOOKUP(K2,Scoring!$A:$B,2,0))+IF(M2="y",1,0)+IF(N2="y",1,0)+IF(O2="y",1,0)+IF(P2="y",1,0),0)</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="R2" s="16"/>
       <c r="S2" s="17"/>
@@ -3424,8 +3411,12 @@
       <c r="C3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
+      <c r="D3" s="24">
+        <v>3.0</v>
+      </c>
+      <c r="E3" s="25">
+        <v>2.0</v>
+      </c>
       <c r="F3" s="26" t="s">
         <v>128</v>
       </c>
@@ -3440,10 +3431,14 @@
       </c>
       <c r="J3" s="99">
         <f>IFERROR((VLOOKUP(D3,Scoring!$A:$B,2,0))+IF(F3="y",1,0)+IF(G3="y",1,0)+IF(H3="y",1,0)+IF(I3="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K3" s="24"/>
-      <c r="L3" s="25"/>
+        <v>15</v>
+      </c>
+      <c r="K3" s="24">
+        <v>4.0</v>
+      </c>
+      <c r="L3" s="25">
+        <v>4.0</v>
+      </c>
       <c r="M3" s="26" t="s">
         <v>128</v>
       </c>
@@ -3458,7 +3453,7 @@
       </c>
       <c r="Q3" s="99">
         <f>IFERROR((VLOOKUP(K3,Scoring!$A:$B,2,0))+IF(M3="y",1,0)+IF(N3="y",1,0)+IF(O3="y",1,0)+IF(P3="y",1,0),0)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="R3" s="24"/>
       <c r="S3" s="25"/>
@@ -3726,8 +3721,12 @@
       <c r="C4" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="36"/>
-      <c r="E4" s="37"/>
+      <c r="D4" s="36">
+        <v>1.0</v>
+      </c>
+      <c r="E4" s="37">
+        <v>3.0</v>
+      </c>
       <c r="F4" s="38" t="s">
         <v>128</v>
       </c>
@@ -3742,10 +3741,14 @@
       </c>
       <c r="J4" s="85">
         <f>IFERROR((VLOOKUP(D4,Scoring!$A:$B,2,0))+IF(F4="y",1,0)+IF(G4="y",1,0)+IF(H4="y",1,0)+IF(I4="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K4" s="36"/>
-      <c r="L4" s="37"/>
+        <v>25</v>
+      </c>
+      <c r="K4" s="36">
+        <v>5.0</v>
+      </c>
+      <c r="L4" s="37">
+        <v>5.0</v>
+      </c>
       <c r="M4" s="38" t="s">
         <v>128</v>
       </c>
@@ -3760,7 +3763,7 @@
       </c>
       <c r="Q4" s="85">
         <f>IFERROR((VLOOKUP(K4,Scoring!$A:$B,2,0))+IF(M4="y",1,0)+IF(N4="y",1,0)+IF(O4="y",1,0)+IF(P4="y",1,0),0)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R4" s="36"/>
       <c r="S4" s="37"/>
@@ -4028,8 +4031,12 @@
       <c r="C5" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="48"/>
-      <c r="E5" s="49"/>
+      <c r="D5" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="E5" s="49">
+        <v>4.0</v>
+      </c>
       <c r="F5" s="50" t="s">
         <v>128</v>
       </c>
@@ -4044,10 +4051,14 @@
       </c>
       <c r="J5" s="99">
         <f>IFERROR((VLOOKUP(D5,Scoring!$A:$B,2,0))+IF(F5="y",1,0)+IF(G5="y",1,0)+IF(H5="y",1,0)+IF(I5="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K5" s="48"/>
-      <c r="L5" s="49"/>
+        <v>12</v>
+      </c>
+      <c r="K5" s="48">
+        <v>6.0</v>
+      </c>
+      <c r="L5" s="49">
+        <v>6.0</v>
+      </c>
       <c r="M5" s="50" t="s">
         <v>128</v>
       </c>
@@ -4062,7 +4073,7 @@
       </c>
       <c r="Q5" s="99">
         <f>IFERROR((VLOOKUP(K5,Scoring!$A:$B,2,0))+IF(M5="y",1,0)+IF(N5="y",1,0)+IF(O5="y",1,0)+IF(P5="y",1,0),0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="R5" s="48"/>
       <c r="S5" s="49"/>
@@ -4330,8 +4341,12 @@
       <c r="C6" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="25"/>
+      <c r="D6" s="24">
+        <v>6.0</v>
+      </c>
+      <c r="E6" s="25">
+        <v>5.0</v>
+      </c>
       <c r="F6" s="26" t="s">
         <v>128</v>
       </c>
@@ -4346,10 +4361,14 @@
       </c>
       <c r="J6" s="85">
         <f>IFERROR((VLOOKUP(D6,Scoring!$A:$B,2,0))+IF(F6="y",1,0)+IF(G6="y",1,0)+IF(H6="y",1,0)+IF(I6="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K6" s="24"/>
-      <c r="L6" s="25"/>
+        <v>8</v>
+      </c>
+      <c r="K6" s="24">
+        <v>11.0</v>
+      </c>
+      <c r="L6" s="25">
+        <v>10.0</v>
+      </c>
       <c r="M6" s="26" t="s">
         <v>128</v>
       </c>
@@ -4364,7 +4383,7 @@
       </c>
       <c r="Q6" s="85">
         <f>IFERROR((VLOOKUP(K6,Scoring!$A:$B,2,0))+IF(M6="y",1,0)+IF(N6="y",1,0)+IF(O6="y",1,0)+IF(P6="y",1,0),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" s="24"/>
       <c r="S6" s="25"/>
@@ -4632,8 +4651,12 @@
       <c r="C7" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="25"/>
+      <c r="D7" s="24">
+        <v>5.0</v>
+      </c>
+      <c r="E7" s="25">
+        <v>6.0</v>
+      </c>
       <c r="F7" s="26" t="s">
         <v>128</v>
       </c>
@@ -4648,10 +4671,14 @@
       </c>
       <c r="J7" s="99">
         <f>IFERROR((VLOOKUP(D7,Scoring!$A:$B,2,0))+IF(F7="y",1,0)+IF(G7="y",1,0)+IF(H7="y",1,0)+IF(I7="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="24"/>
-      <c r="L7" s="25"/>
+        <v>10</v>
+      </c>
+      <c r="K7" s="24">
+        <v>10.0</v>
+      </c>
+      <c r="L7" s="25">
+        <v>11.0</v>
+      </c>
       <c r="M7" s="26" t="s">
         <v>128</v>
       </c>
@@ -4666,7 +4693,7 @@
       </c>
       <c r="Q7" s="99">
         <f>IFERROR((VLOOKUP(K7,Scoring!$A:$B,2,0))+IF(M7="y",1,0)+IF(N7="y",1,0)+IF(O7="y",1,0)+IF(P7="y",1,0),0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R7" s="24"/>
       <c r="S7" s="25"/>
@@ -4934,8 +4961,12 @@
       <c r="C8" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="36"/>
-      <c r="E8" s="37"/>
+      <c r="D8" s="36">
+        <v>7.0</v>
+      </c>
+      <c r="E8" s="37">
+        <v>7.0</v>
+      </c>
       <c r="F8" s="38" t="s">
         <v>128</v>
       </c>
@@ -4950,10 +4981,14 @@
       </c>
       <c r="J8" s="85">
         <f>IFERROR((VLOOKUP(D8,Scoring!$A:$B,2,0))+IF(F8="y",1,0)+IF(G8="y",1,0)+IF(H8="y",1,0)+IF(I8="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K8" s="36"/>
-      <c r="L8" s="37"/>
+        <v>6</v>
+      </c>
+      <c r="K8" s="36">
+        <v>2.0</v>
+      </c>
+      <c r="L8" s="37">
+        <v>1.0</v>
+      </c>
       <c r="M8" s="38" t="s">
         <v>128</v>
       </c>
@@ -4968,7 +5003,7 @@
       </c>
       <c r="Q8" s="85">
         <f>IFERROR((VLOOKUP(K8,Scoring!$A:$B,2,0))+IF(M8="y",1,0)+IF(N8="y",1,0)+IF(O8="y",1,0)+IF(P8="y",1,0),0)</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="R8" s="36"/>
       <c r="S8" s="37"/>
@@ -5236,8 +5271,12 @@
       <c r="C9" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="48"/>
-      <c r="E9" s="49"/>
+      <c r="D9" s="48">
+        <v>8.0</v>
+      </c>
+      <c r="E9" s="49">
+        <v>8.0</v>
+      </c>
       <c r="F9" s="50" t="s">
         <v>128</v>
       </c>
@@ -5252,10 +5291,14 @@
       </c>
       <c r="J9" s="99">
         <f>IFERROR((VLOOKUP(D9,Scoring!$A:$B,2,0))+IF(F9="y",1,0)+IF(G9="y",1,0)+IF(H9="y",1,0)+IF(I9="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K9" s="48"/>
-      <c r="L9" s="49"/>
+        <v>4</v>
+      </c>
+      <c r="K9" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="L9" s="49">
+        <v>2.0</v>
+      </c>
       <c r="M9" s="50" t="s">
         <v>128</v>
       </c>
@@ -5270,7 +5313,7 @@
       </c>
       <c r="Q9" s="99">
         <f>IFERROR((VLOOKUP(K9,Scoring!$A:$B,2,0))+IF(M9="y",1,0)+IF(N9="y",1,0)+IF(O9="y",1,0)+IF(P9="y",1,0),0)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="R9" s="48"/>
       <c r="S9" s="49"/>
@@ -5538,8 +5581,12 @@
       <c r="C10" s="15" t="s">
         <v>397</v>
       </c>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25"/>
+      <c r="D10" s="24">
+        <v>9.0</v>
+      </c>
+      <c r="E10" s="25">
+        <v>9.0</v>
+      </c>
       <c r="F10" s="26" t="s">
         <v>128</v>
       </c>
@@ -5554,10 +5601,14 @@
       </c>
       <c r="J10" s="85">
         <f>IFERROR((VLOOKUP(D10,Scoring!$A:$B,2,0))+IF(F10="y",1,0)+IF(G10="y",1,0)+IF(H10="y",1,0)+IF(I10="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="24"/>
-      <c r="L10" s="25"/>
+        <v>3</v>
+      </c>
+      <c r="K10" s="24">
+        <v>7.0</v>
+      </c>
+      <c r="L10" s="25">
+        <v>9.0</v>
+      </c>
       <c r="M10" s="26" t="s">
         <v>128</v>
       </c>
@@ -5572,7 +5623,7 @@
       </c>
       <c r="Q10" s="85">
         <f>IFERROR((VLOOKUP(K10,Scoring!$A:$B,2,0))+IF(M10="y",1,0)+IF(N10="y",1,0)+IF(O10="y",1,0)+IF(P10="y",1,0),0)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R10" s="24"/>
       <c r="S10" s="25"/>
@@ -5840,8 +5891,12 @@
       <c r="C11" s="15" t="s">
         <v>397</v>
       </c>
-      <c r="D11" s="24"/>
-      <c r="E11" s="25"/>
+      <c r="D11" s="24">
+        <v>10.0</v>
+      </c>
+      <c r="E11" s="25">
+        <v>10.0</v>
+      </c>
       <c r="F11" s="26" t="s">
         <v>128</v>
       </c>
@@ -5856,10 +5911,14 @@
       </c>
       <c r="J11" s="99">
         <f>IFERROR((VLOOKUP(D11,Scoring!$A:$B,2,0))+IF(F11="y",1,0)+IF(G11="y",1,0)+IF(H11="y",1,0)+IF(I11="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="24"/>
-      <c r="L11" s="25"/>
+        <v>2</v>
+      </c>
+      <c r="K11" s="24">
+        <v>8.0</v>
+      </c>
+      <c r="L11" s="25">
+        <v>7.0</v>
+      </c>
       <c r="M11" s="26" t="s">
         <v>128</v>
       </c>
@@ -5874,7 +5933,7 @@
       </c>
       <c r="Q11" s="99">
         <f>IFERROR((VLOOKUP(K11,Scoring!$A:$B,2,0))+IF(M11="y",1,0)+IF(N11="y",1,0)+IF(O11="y",1,0)+IF(P11="y",1,0),0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R11" s="24"/>
       <c r="S11" s="25"/>
@@ -6142,8 +6201,12 @@
       <c r="C12" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="36"/>
-      <c r="E12" s="37"/>
+      <c r="D12" s="36">
+        <v>11.0</v>
+      </c>
+      <c r="E12" s="37">
+        <v>11.0</v>
+      </c>
       <c r="F12" s="38" t="s">
         <v>128</v>
       </c>
@@ -6158,10 +6221,14 @@
       </c>
       <c r="J12" s="85">
         <f>IFERROR((VLOOKUP(D12,Scoring!$A:$B,2,0))+IF(F12="y",1,0)+IF(G12="y",1,0)+IF(H12="y",1,0)+IF(I12="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K12" s="36"/>
-      <c r="L12" s="37"/>
+        <v>1</v>
+      </c>
+      <c r="K12" s="36">
+        <v>9.0</v>
+      </c>
+      <c r="L12" s="37">
+        <v>8.0</v>
+      </c>
       <c r="M12" s="38" t="s">
         <v>128</v>
       </c>
@@ -6176,7 +6243,7 @@
       </c>
       <c r="Q12" s="85">
         <f>IFERROR((VLOOKUP(K12,Scoring!$A:$B,2,0))+IF(M12="y",1,0)+IF(N12="y",1,0)+IF(O12="y",1,0)+IF(P12="y",1,0),0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R12" s="36"/>
       <c r="S12" s="37"/>
@@ -6444,8 +6511,12 @@
       <c r="C13" s="15" t="s">
         <v>397</v>
       </c>
-      <c r="D13" s="24"/>
-      <c r="E13" s="25"/>
+      <c r="D13" s="24">
+        <v>12.0</v>
+      </c>
+      <c r="E13" s="25">
+        <v>12.0</v>
+      </c>
       <c r="F13" s="26" t="s">
         <v>128</v>
       </c>
@@ -6460,10 +6531,14 @@
       </c>
       <c r="J13" s="99">
         <f>IFERROR((VLOOKUP(D13,Scoring!$A:$B,2,0))+IF(F13="y",1,0)+IF(G13="y",1,0)+IF(H13="y",1,0)+IF(I13="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K13" s="24"/>
-      <c r="L13" s="25"/>
+        <v>1</v>
+      </c>
+      <c r="K13" s="24">
+        <v>12.0</v>
+      </c>
+      <c r="L13" s="25">
+        <v>12.0</v>
+      </c>
       <c r="M13" s="26" t="s">
         <v>128</v>
       </c>
@@ -6478,7 +6553,7 @@
       </c>
       <c r="Q13" s="99">
         <f>IFERROR((VLOOKUP(K13,Scoring!$A:$B,2,0))+IF(M13="y",1,0)+IF(N13="y",1,0)+IF(O13="y",1,0)+IF(P13="y",1,0),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R13" s="24"/>
       <c r="S13" s="25"/>
@@ -6746,8 +6821,12 @@
       <c r="C14" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="36"/>
-      <c r="E14" s="37"/>
+      <c r="D14" s="36">
+        <v>13.0</v>
+      </c>
+      <c r="E14" s="37">
+        <v>13.0</v>
+      </c>
       <c r="F14" s="38" t="s">
         <v>128</v>
       </c>
@@ -6762,10 +6841,14 @@
       </c>
       <c r="J14" s="85">
         <f>IFERROR((VLOOKUP(D14,Scoring!$A:$B,2,0))+IF(F14="y",1,0)+IF(G14="y",1,0)+IF(H14="y",1,0)+IF(I14="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K14" s="36"/>
-      <c r="L14" s="37"/>
+        <v>1</v>
+      </c>
+      <c r="K14" s="36">
+        <v>13.0</v>
+      </c>
+      <c r="L14" s="37">
+        <v>16.0</v>
+      </c>
       <c r="M14" s="38" t="s">
         <v>128</v>
       </c>
@@ -6780,7 +6863,7 @@
       </c>
       <c r="Q14" s="85">
         <f>IFERROR((VLOOKUP(K14,Scoring!$A:$B,2,0))+IF(M14="y",1,0)+IF(N14="y",1,0)+IF(O14="y",1,0)+IF(P14="y",1,0),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" s="36"/>
       <c r="S14" s="37"/>
@@ -7048,8 +7131,12 @@
       <c r="C15" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="48"/>
-      <c r="E15" s="49"/>
+      <c r="D15" s="48">
+        <v>14.0</v>
+      </c>
+      <c r="E15" s="49">
+        <v>14.0</v>
+      </c>
       <c r="F15" s="50" t="s">
         <v>128</v>
       </c>
@@ -7064,10 +7151,14 @@
       </c>
       <c r="J15" s="99">
         <f>IFERROR((VLOOKUP(D15,Scoring!$A:$B,2,0))+IF(F15="y",1,0)+IF(G15="y",1,0)+IF(H15="y",1,0)+IF(I15="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K15" s="48"/>
-      <c r="L15" s="49"/>
+        <v>1</v>
+      </c>
+      <c r="K15" s="48">
+        <v>14.0</v>
+      </c>
+      <c r="L15" s="49">
+        <v>15.0</v>
+      </c>
       <c r="M15" s="50" t="s">
         <v>128</v>
       </c>
@@ -7082,7 +7173,7 @@
       </c>
       <c r="Q15" s="99">
         <f>IFERROR((VLOOKUP(K15,Scoring!$A:$B,2,0))+IF(M15="y",1,0)+IF(N15="y",1,0)+IF(O15="y",1,0)+IF(P15="y",1,0),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R15" s="48"/>
       <c r="S15" s="49"/>
@@ -7350,8 +7441,12 @@
       <c r="C16" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="24"/>
-      <c r="E16" s="25"/>
+      <c r="D16" s="24">
+        <v>15.0</v>
+      </c>
+      <c r="E16" s="25">
+        <v>15.0</v>
+      </c>
       <c r="F16" s="26" t="s">
         <v>128</v>
       </c>
@@ -7366,10 +7461,14 @@
       </c>
       <c r="J16" s="85">
         <f>IFERROR((VLOOKUP(D16,Scoring!$A:$B,2,0))+IF(F16="y",1,0)+IF(G16="y",1,0)+IF(H16="y",1,0)+IF(I16="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K16" s="24"/>
-      <c r="L16" s="25"/>
+        <v>1</v>
+      </c>
+      <c r="K16" s="24">
+        <v>15.0</v>
+      </c>
+      <c r="L16" s="25">
+        <v>14.0</v>
+      </c>
       <c r="M16" s="26" t="s">
         <v>128</v>
       </c>
@@ -7384,7 +7483,7 @@
       </c>
       <c r="Q16" s="85">
         <f>IFERROR((VLOOKUP(K16,Scoring!$A:$B,2,0))+IF(M16="y",1,0)+IF(N16="y",1,0)+IF(O16="y",1,0)+IF(P16="y",1,0),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R16" s="24"/>
       <c r="S16" s="25"/>
@@ -7652,8 +7751,12 @@
       <c r="C17" s="59" t="s">
         <v>397</v>
       </c>
-      <c r="D17" s="60"/>
-      <c r="E17" s="61"/>
+      <c r="D17" s="60">
+        <v>16.0</v>
+      </c>
+      <c r="E17" s="61">
+        <v>16.0</v>
+      </c>
       <c r="F17" s="62" t="s">
         <v>128</v>
       </c>
@@ -7668,10 +7771,14 @@
       </c>
       <c r="J17" s="137">
         <f>IFERROR((VLOOKUP(D17,Scoring!$A:$B,2,0))+IF(F17="y",1,0)+IF(G17="y",1,0)+IF(H17="y",1,0)+IF(I17="y",1,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K17" s="60"/>
-      <c r="L17" s="61"/>
+        <v>1</v>
+      </c>
+      <c r="K17" s="60">
+        <v>16.0</v>
+      </c>
+      <c r="L17" s="61">
+        <v>13.0</v>
+      </c>
       <c r="M17" s="62" t="s">
         <v>128</v>
       </c>
@@ -7686,7 +7793,7 @@
       </c>
       <c r="Q17" s="137">
         <f>IFERROR((VLOOKUP(K17,Scoring!$A:$B,2,0))+IF(M17="y",1,0)+IF(N17="y",1,0)+IF(O17="y",1,0)+IF(P17="y",1,0),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17" s="60"/>
       <c r="S17" s="61"/>
@@ -7978,37 +8085,37 @@
         <v>403</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>292</v>
+        <v>404</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B3" s="69" t="s">
+        <v>406</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>404</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B4" s="69" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>292</v>
+        <v>404</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>407</v>
+        <v>143</v>
       </c>
       <c r="B5" s="69" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>292</v>
@@ -8016,10 +8123,10 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="B6" s="69" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>292</v>
@@ -8027,7 +8134,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>411</v>
+        <v>276</v>
       </c>
       <c r="B7" s="69" t="s">
         <v>412</v>
@@ -8038,10 +8145,10 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>413</v>
+        <v>144</v>
       </c>
       <c r="B8" s="69" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>292</v>
@@ -8049,10 +8156,10 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>415</v>
+        <v>151</v>
       </c>
       <c r="B9" s="69" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>292</v>
@@ -8060,10 +8167,10 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>417</v>
+        <v>149</v>
       </c>
       <c r="B10" s="69" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>292</v>
@@ -8071,10 +8178,10 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>419</v>
+        <v>157</v>
       </c>
       <c r="B11" s="69" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>292</v>
@@ -8082,10 +8189,10 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="B12" s="69" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>292</v>
@@ -8093,10 +8200,10 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>423</v>
+        <v>148</v>
       </c>
       <c r="B13" s="69" t="s">
-        <v>424</v>
+        <v>417</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>292</v>
@@ -8104,10 +8211,10 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>425</v>
+        <v>153</v>
       </c>
       <c r="B14" s="69" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>292</v>
@@ -8115,10 +8222,10 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>427</v>
+        <v>159</v>
       </c>
       <c r="B15" s="69" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>292</v>
@@ -8126,10 +8233,10 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>429</v>
+        <v>141</v>
       </c>
       <c r="B16" s="69" t="s">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>292</v>
@@ -8137,10 +8244,10 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B17" s="69" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>292</v>
@@ -8148,10 +8255,10 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>154</v>
+        <v>422</v>
       </c>
       <c r="B18" s="69" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>292</v>
@@ -8159,10 +8266,10 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>432</v>
+        <v>150</v>
       </c>
       <c r="B19" s="69" t="s">
-        <v>433</v>
+        <v>423</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>292</v>
@@ -8170,10 +8277,10 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B20" s="69" t="s">
-        <v>433</v>
+        <v>424</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>292</v>
@@ -8181,12 +8288,34 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="B21" s="69" t="s">
+        <v>426</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B22" s="69" t="s">
+        <v>426</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="B21" s="69" t="s">
-        <v>434</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="B23" s="69" t="s">
+        <v>427</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>292</v>
       </c>
     </row>

</xml_diff>